<commit_message>
updated spreadsheet for sensor circuitry
</commit_message>
<xml_diff>
--- a/Excel/sensors.xlsx
+++ b/Excel/sensors.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\University\Engineering\Stage3\Semester2\ELECTENG 311\311\Excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d393d29289b0eecc/Documents/School Stuff/ELECTENG 311/311/Excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEF83167-29AA-4D2C-9F19-8FB03B27FB56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="135" documentId="13_ncr:1_{FEF83167-29AA-4D2C-9F19-8FB03B27FB56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{12279AB5-856C-4769-9720-6B7ED887E860}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Current Sensor" sheetId="1" r:id="rId1"/>
@@ -136,7 +136,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="143">
   <si>
     <t>Current Sense Amplifier</t>
   </si>
@@ -324,9 +324,6 @@
     <t>(I_high)^2 * (R1 + R_temp_high)</t>
   </si>
   <si>
-    <t>R_temp_low (-15°C)</t>
-  </si>
-  <si>
     <t>10 k * (R_t / R_25)</t>
   </si>
   <si>
@@ -336,9 +333,6 @@
     <t>Vcc / (R_temp_low + R1)</t>
   </si>
   <si>
-    <t>R_temp_high (80°C)</t>
-  </si>
-  <si>
     <t>I_high (80°C)</t>
   </si>
   <si>
@@ -414,15 +408,9 @@
     <t>Test value for simulations</t>
   </si>
   <si>
-    <t>Vv_min</t>
-  </si>
-  <si>
     <t>Minimum super cap voltage</t>
   </si>
   <si>
-    <t>Vv_max</t>
-  </si>
-  <si>
     <t>Maximum super cap voltage</t>
   </si>
   <si>
@@ -430,9 +418,6 @@
   </si>
   <si>
     <t>1 / (2*pi*R1*C1)</t>
-  </si>
-  <si>
-    <t>(kΩ)</t>
   </si>
   <si>
     <t>Min (A)</t>
@@ -558,17 +543,81 @@
   <si>
     <t>Here the snesor output voltage is chosen, then the temperature is determined. Kind of reverse of the above.</t>
   </si>
+  <si>
+    <t>(Ω)</t>
+  </si>
+  <si>
+    <t>Current through reference voltage divider</t>
+  </si>
+  <si>
+    <t>Max power dissipated</t>
+  </si>
+  <si>
+    <t>(aim for well under 0.125 W, from 209 slides)</t>
+  </si>
+  <si>
+    <t>R_temp_low (-10°C)</t>
+  </si>
+  <si>
+    <t>R_temp_high (70°C)</t>
+  </si>
+  <si>
+    <t>Note: cap is rated from 2.5V to 3.8V</t>
+  </si>
+  <si>
+    <t>5V *  Rb / (Ra + Rb)</t>
+  </si>
+  <si>
+    <t>Ra</t>
+  </si>
+  <si>
+    <t>Rb</t>
+  </si>
+  <si>
+    <t>Low output</t>
+  </si>
+  <si>
+    <t>Rf</t>
+  </si>
+  <si>
+    <t>Ri</t>
+  </si>
+  <si>
+    <t>kΩ</t>
+  </si>
+  <si>
+    <t>Vsc_min</t>
+  </si>
+  <si>
+    <t>Vsc_max</t>
+  </si>
+  <si>
+    <t>(1 + Rf/Ri) * Vsc_min - Rf/Ri * Vos</t>
+  </si>
+  <si>
+    <t>Vos (voltage across Rb)</t>
+  </si>
+  <si>
+    <t>High output</t>
+  </si>
+  <si>
+    <t>(1 + Rf/Ri) * Vsc_max - Rf/Ri * Vos</t>
+  </si>
+  <si>
+    <t>Note: output calculations assume amplifier circuit has negligible loading on the voltage reference divider.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="0.000000"/>
     <numFmt numFmtId="165" formatCode="0.000E+00"/>
     <numFmt numFmtId="166" formatCode="0.000"/>
+    <numFmt numFmtId="169" formatCode="0.0000E+00"/>
   </numFmts>
-  <fonts count="16" x14ac:knownFonts="1">
+  <fonts count="17" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -680,6 +729,14 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -707,7 +764,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -778,6 +835,12 @@
     <xf numFmtId="1" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -793,10 +856,10 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="169" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -930,23 +993,119 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>57150</xdr:colOff>
-      <xdr:row>8</xdr:row>
-      <xdr:rowOff>95250</xdr:rowOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>152400</xdr:colOff>
-      <xdr:row>21</xdr:row>
-      <xdr:rowOff>342900</xdr:rowOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>304800</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="3073" name="AutoShape 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4927A03D-9F93-A97F-DCAB-3B71BB6F1F75}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="10706100" y="3305175"/>
+          <a:ext cx="304800" cy="304800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>304800</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="3074" name="AutoShape 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D92EE29D-0911-5A22-D1F8-8A8FD971799E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="10706100" y="9629775"/>
+          <a:ext cx="304800" cy="304800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>333375</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>1738312</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>507999</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>71436</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="8" name="Picture 7">
+        <xdr:cNvPr id="3" name="Picture 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0B454C22-703E-E42A-236D-E42CA9732861}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AFBEC82D-4E3B-0F52-EEFF-0687F3FE6863}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -955,7 +1114,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
               <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
@@ -968,8 +1127,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2838450" y="5067300"/>
-          <a:ext cx="11449050" cy="5943600"/>
+          <a:off x="12882563" y="1738312"/>
+          <a:ext cx="10699749" cy="8024812"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1494,26 +1653,26 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B1:Q14"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="35.25" customHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="35.25" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="40.6640625" style="2" customWidth="1"/>
-    <col min="2" max="2" width="67.33203125" style="2" customWidth="1"/>
-    <col min="3" max="3" width="38.6640625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="18.6640625" style="2" customWidth="1"/>
-    <col min="5" max="7" width="9.109375" style="2"/>
-    <col min="8" max="9" width="38.6640625" style="2" customWidth="1"/>
-    <col min="10" max="10" width="18.6640625" style="2" customWidth="1"/>
-    <col min="11" max="13" width="9.109375" style="2"/>
-    <col min="14" max="14" width="47.6640625" style="2" customWidth="1"/>
-    <col min="15" max="15" width="76.109375" style="2" customWidth="1"/>
-    <col min="16" max="16" width="18.6640625" style="2" customWidth="1"/>
-    <col min="17" max="16384" width="9.109375" style="2"/>
+    <col min="1" max="1" width="40.7109375" style="2" customWidth="1"/>
+    <col min="2" max="2" width="67.28515625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="38.7109375" style="2" customWidth="1"/>
+    <col min="4" max="4" width="18.7109375" style="2" customWidth="1"/>
+    <col min="5" max="7" width="9.140625" style="2"/>
+    <col min="8" max="9" width="38.7109375" style="2" customWidth="1"/>
+    <col min="10" max="10" width="18.7109375" style="2" customWidth="1"/>
+    <col min="11" max="13" width="9.140625" style="2"/>
+    <col min="14" max="14" width="47.7109375" style="2" customWidth="1"/>
+    <col min="15" max="15" width="76.140625" style="2" customWidth="1"/>
+    <col min="16" max="16" width="18.7109375" style="2" customWidth="1"/>
+    <col min="17" max="16384" width="9.140625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:17" ht="150" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:17" ht="150" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B1" s="7"/>
     </row>
-    <row r="2" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="10" t="s">
         <v>0</v>
       </c>
@@ -1537,7 +1696,7 @@
       <c r="J2" s="1"/>
       <c r="K2" s="1"/>
     </row>
-    <row r="3" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
@@ -1549,27 +1708,27 @@
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
     </row>
-    <row r="4" spans="2:17" ht="73.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="B4" s="24"/>
-      <c r="C4" s="24"/>
-      <c r="D4" s="24"/>
-      <c r="E4" s="24"/>
+    <row r="4" spans="2:17" ht="73.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B4" s="26"/>
+      <c r="C4" s="26"/>
+      <c r="D4" s="26"/>
+      <c r="E4" s="26"/>
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
-      <c r="H4" s="26" t="s">
+      <c r="H4" s="28" t="s">
         <v>4</v>
       </c>
-      <c r="I4" s="27"/>
-      <c r="J4" s="27"/>
-      <c r="K4" s="27"/>
-      <c r="N4" s="25" t="s">
+      <c r="I4" s="29"/>
+      <c r="J4" s="29"/>
+      <c r="K4" s="29"/>
+      <c r="N4" s="27" t="s">
         <v>5</v>
       </c>
-      <c r="O4" s="25"/>
-      <c r="P4" s="25"/>
-      <c r="Q4" s="25"/>
-    </row>
-    <row r="5" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="O4" s="27"/>
+      <c r="P4" s="27"/>
+      <c r="Q4" s="27"/>
+    </row>
+    <row r="5" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="10" t="s">
         <v>6</v>
       </c>
@@ -1609,7 +1768,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="1" t="s">
         <v>10</v>
       </c>
@@ -1632,7 +1791,7 @@
       </c>
       <c r="J6" s="1">
         <f>D7*D10</f>
-        <v>-1.4999999999999999E-2</v>
+        <v>-1.7340000000000001E-2</v>
       </c>
       <c r="K6" s="1" t="s">
         <v>12</v>
@@ -1645,13 +1804,13 @@
       </c>
       <c r="P6" s="2">
         <f>POWER(D7,2)*D10</f>
-        <v>2.2499999999999999E-2</v>
+        <v>4.4217000000000006E-3</v>
       </c>
       <c r="Q6" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="1" t="s">
         <v>18</v>
       </c>
@@ -1659,7 +1818,7 @@
         <v>11</v>
       </c>
       <c r="D7" s="1">
-        <v>-1.5</v>
+        <v>-0.255</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>19</v>
@@ -1674,7 +1833,7 @@
       </c>
       <c r="J7" s="1">
         <f>D8*D10</f>
-        <v>1.4999999999999999E-2</v>
+        <v>1.7340000000000001E-2</v>
       </c>
       <c r="K7" s="1" t="s">
         <v>12</v>
@@ -1687,13 +1846,13 @@
       </c>
       <c r="P7" s="2">
         <f>POWER(D8,2)*D10</f>
-        <v>2.2499999999999999E-2</v>
+        <v>4.4217000000000006E-3</v>
       </c>
       <c r="Q7" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="1" t="s">
         <v>24</v>
       </c>
@@ -1701,7 +1860,7 @@
         <v>11</v>
       </c>
       <c r="D8" s="1">
-        <v>1.5</v>
+        <v>0.255</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>19</v>
@@ -1716,7 +1875,7 @@
       </c>
       <c r="J8" s="8">
         <f>E2*J6+D9</f>
-        <v>1</v>
+        <v>0.76599999999999979</v>
       </c>
       <c r="K8" s="8" t="s">
         <v>12</v>
@@ -1729,13 +1888,13 @@
       </c>
       <c r="P8" s="2">
         <f>(J13 * 100)/(ABS(J7) * POWER(10, (I2 / 20)))</f>
-        <v>2.3283333333333333E-2</v>
+        <v>2.0134544405997691E-2</v>
       </c>
       <c r="Q8" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="9" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="1" t="s">
         <v>30</v>
       </c>
@@ -1758,7 +1917,7 @@
       </c>
       <c r="J9" s="8">
         <f>E2*J7+D9</f>
-        <v>4</v>
+        <v>4.234</v>
       </c>
       <c r="K9" s="8" t="s">
         <v>12</v>
@@ -1771,13 +1930,13 @@
       </c>
       <c r="P9" s="2">
         <f>(J14 * 100)/(ABS(J6) * POWER(10, (I2 / 20)))</f>
-        <v>2.3383333333333332E-2</v>
+        <v>2.0234544405997694E-2</v>
       </c>
       <c r="Q9" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="10" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="1" t="s">
         <v>35</v>
       </c>
@@ -1785,7 +1944,7 @@
         <v>11</v>
       </c>
       <c r="D10" s="1">
-        <v>0.01</v>
+        <v>6.8000000000000005E-2</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>36</v>
@@ -1806,7 +1965,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
       <c r="D11" s="4"/>
@@ -1819,13 +1978,13 @@
       </c>
       <c r="J11" s="2">
         <f>D6 - J7</f>
-        <v>3.4849999999999999</v>
+        <v>3.4826600000000001</v>
       </c>
       <c r="K11" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="4"/>
       <c r="C12" s="4"/>
       <c r="D12" s="4"/>
@@ -1838,13 +1997,13 @@
       </c>
       <c r="J12" s="2">
         <f>D6 - J6</f>
-        <v>3.5150000000000001</v>
+        <v>3.5173399999999999</v>
       </c>
       <c r="K12" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="H13" s="1" t="s">
         <v>43</v>
       </c>
@@ -1853,13 +2012,13 @@
       </c>
       <c r="J13" s="2">
         <f>(J10 + J11) / 2</f>
-        <v>3.4924999999999997</v>
+        <v>3.49133</v>
       </c>
       <c r="K13" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="H14" s="2" t="s">
         <v>45</v>
       </c>
@@ -1868,7 +2027,7 @@
       </c>
       <c r="J14" s="2">
         <f>(J10 + J12) / 2</f>
-        <v>3.5075000000000003</v>
+        <v>3.50867</v>
       </c>
       <c r="K14" s="2" t="s">
         <v>12</v>
@@ -1888,28 +2047,28 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F2E2C88-472F-40E6-9BB7-0CE3D1C9A840}">
   <dimension ref="B1:Q17"/>
-  <sheetFormatPr defaultRowHeight="35.25" customHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="35.25" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="40.6640625" style="5" customWidth="1"/>
-    <col min="2" max="2" width="58.6640625" style="5" customWidth="1"/>
-    <col min="3" max="3" width="33.88671875" style="5" customWidth="1"/>
-    <col min="4" max="4" width="17.5546875" style="5" customWidth="1"/>
-    <col min="5" max="5" width="9.6640625" style="5" customWidth="1"/>
-    <col min="6" max="7" width="9.109375" style="5" customWidth="1"/>
-    <col min="8" max="8" width="34.44140625" style="5" customWidth="1"/>
-    <col min="9" max="9" width="40.88671875" style="5" customWidth="1"/>
-    <col min="10" max="10" width="25.44140625" style="5" customWidth="1"/>
-    <col min="11" max="11" width="9.6640625" style="5" customWidth="1"/>
-    <col min="12" max="13" width="9.109375" style="5" customWidth="1"/>
-    <col min="14" max="14" width="34.44140625" style="5" customWidth="1"/>
-    <col min="15" max="15" width="52.88671875" style="5" customWidth="1"/>
-    <col min="16" max="16" width="17.5546875" style="5" customWidth="1"/>
-    <col min="17" max="17" width="34.44140625" style="5" customWidth="1"/>
-    <col min="18" max="16380" width="9.109375" style="5" customWidth="1"/>
-    <col min="16381" max="16384" width="9.109375" style="5"/>
+    <col min="1" max="1" width="40.7109375" style="5" customWidth="1"/>
+    <col min="2" max="2" width="58.7109375" style="5" customWidth="1"/>
+    <col min="3" max="3" width="33.85546875" style="5" customWidth="1"/>
+    <col min="4" max="4" width="17.5703125" style="5" customWidth="1"/>
+    <col min="5" max="5" width="9.7109375" style="5" customWidth="1"/>
+    <col min="6" max="7" width="9.140625" style="5" customWidth="1"/>
+    <col min="8" max="8" width="34.42578125" style="5" customWidth="1"/>
+    <col min="9" max="9" width="40.85546875" style="5" customWidth="1"/>
+    <col min="10" max="10" width="25.42578125" style="5" customWidth="1"/>
+    <col min="11" max="11" width="9.7109375" style="5" customWidth="1"/>
+    <col min="12" max="13" width="9.140625" style="5" customWidth="1"/>
+    <col min="14" max="14" width="34.42578125" style="5" customWidth="1"/>
+    <col min="15" max="15" width="52.85546875" style="5" customWidth="1"/>
+    <col min="16" max="16" width="17.5703125" style="5" customWidth="1"/>
+    <col min="17" max="17" width="34.42578125" style="5" customWidth="1"/>
+    <col min="18" max="16380" width="9.140625" style="5" customWidth="1"/>
+    <col min="16381" max="16384" width="9.140625" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:17" ht="150" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:17" ht="150" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -1927,7 +2086,7 @@
       <c r="P1" s="1"/>
       <c r="Q1" s="1"/>
     </row>
-    <row r="2" spans="2:17" ht="57.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:17" ht="57.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="10" t="s">
         <v>47</v>
       </c>
@@ -1953,7 +2112,7 @@
       <c r="P2" s="1"/>
       <c r="Q2" s="1"/>
     </row>
-    <row r="4" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="10" t="s">
         <v>6</v>
       </c>
@@ -1995,7 +2154,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="2:17" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:17" ht="69.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="1" t="s">
         <v>51</v>
       </c>
@@ -2018,7 +2177,7 @@
       </c>
       <c r="J5" s="13">
         <f>(D5*D8) / (D8 + D6)</f>
-        <v>0.48234953965141808</v>
+        <v>0.77427888069098993</v>
       </c>
       <c r="K5" s="1" t="s">
         <v>12</v>
@@ -2031,15 +2190,15 @@
       <c r="O5" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="P5" s="14">
+      <c r="P5" s="31">
         <f>POWER(J7,2)*(D5+D7)</f>
-        <v>2.3654745406422815E-4</v>
+        <v>3.3903900917282403E-4</v>
       </c>
       <c r="Q5" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="2:17" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:17" ht="69.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="1" t="s">
         <v>56</v>
       </c>
@@ -2062,7 +2221,7 @@
       </c>
       <c r="J6" s="13">
         <f>(D5*D7) / (D7 + D6)</f>
-        <v>4.4709554544492649</v>
+        <v>4.1911348378225348</v>
       </c>
       <c r="K6" s="1" t="s">
         <v>12</v>
@@ -2075,23 +2234,23 @@
       <c r="O6" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="P6" s="14">
+      <c r="P6" s="31">
         <f>POWER(J8, 2) * (D6+D8)</f>
-        <v>2.258825230174291E-3</v>
+        <v>2.1128605596545053E-3</v>
       </c>
       <c r="Q6" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="C7" s="1" t="s">
-        <v>63</v>
-      </c>
       <c r="D7" s="1">
-        <v>84510</v>
+        <v>51815</v>
       </c>
       <c r="E7" s="6" t="s">
         <v>36</v>
@@ -2099,14 +2258,14 @@
       <c r="F7" s="1"/>
       <c r="G7" s="1"/>
       <c r="H7" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="I7" s="1" t="s">
         <v>64</v>
-      </c>
-      <c r="I7" s="1" t="s">
-        <v>65</v>
       </c>
       <c r="J7" s="13">
         <f>D5 / (D7 + D6)</f>
-        <v>5.290445455507354E-5</v>
+        <v>8.0886516217746498E-5</v>
       </c>
       <c r="K7" s="1" t="s">
         <v>19</v>
@@ -2118,15 +2277,15 @@
       <c r="P7" s="1"/>
       <c r="Q7" s="1"/>
     </row>
-    <row r="8" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="1" t="s">
-        <v>66</v>
+        <v>127</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D8" s="1">
-        <v>1067.7</v>
+        <v>1832.3</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>36</v>
@@ -2134,14 +2293,14 @@
       <c r="F8" s="1"/>
       <c r="G8" s="1"/>
       <c r="H8" s="1" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="J8" s="13">
         <f>D5 / (D8 + D6)</f>
-        <v>4.5176504603485819E-4</v>
+        <v>4.2257211193090104E-4</v>
       </c>
       <c r="K8" s="1" t="s">
         <v>19</v>
@@ -2153,7 +2312,7 @@
       <c r="P8" s="1"/>
       <c r="Q8" s="1"/>
     </row>
-    <row r="9" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
       <c r="D9" s="1"/>
@@ -2171,7 +2330,7 @@
       <c r="P9" s="1"/>
       <c r="Q9" s="1"/>
     </row>
-    <row r="10" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
@@ -2189,15 +2348,15 @@
       <c r="P10" s="10"/>
       <c r="Q10" s="10"/>
     </row>
-    <row r="11" spans="2:17" ht="99.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="N11" s="30" t="s">
-        <v>126</v>
-      </c>
-      <c r="O11" s="30"/>
-      <c r="P11" s="30"/>
-      <c r="Q11" s="30"/>
-    </row>
-    <row r="12" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:17" ht="99.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="N11" s="25" t="s">
+        <v>121</v>
+      </c>
+      <c r="O11" s="25"/>
+      <c r="P11" s="25"/>
+      <c r="Q11" s="25"/>
+    </row>
+    <row r="12" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="N12" s="10" t="s">
         <v>6</v>
       </c>
@@ -2211,12 +2370,12 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="N13" s="1" t="s">
         <v>51</v>
       </c>
       <c r="O13" s="1" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="P13" s="5">
         <v>5</v>
@@ -2225,7 +2384,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="N14" s="1" t="s">
         <v>56</v>
       </c>
@@ -2236,12 +2395,12 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="15" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="N15" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="O15" s="1" t="s">
         <v>119</v>
-      </c>
-      <c r="O15" s="1" t="s">
-        <v>124</v>
       </c>
       <c r="P15" s="5">
         <v>10000</v>
@@ -2250,13 +2409,13 @@
         <v>36</v>
       </c>
     </row>
-    <row r="16" spans="2:17" ht="34.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:17" ht="34.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I16" s="1"/>
       <c r="N16" s="1" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="O16" s="1" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="P16" s="5">
         <v>4.5</v>
@@ -2265,19 +2424,19 @@
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="14:17" ht="72.599999999999994" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="14:17" ht="72.599999999999994" customHeight="1" x14ac:dyDescent="0.25">
       <c r="N17" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="O17" s="29" t="s">
-        <v>121</v>
+        <v>115</v>
+      </c>
+      <c r="O17" s="24" t="s">
+        <v>116</v>
       </c>
       <c r="P17" s="5">
         <f>(-1*P16*P14)/(P15*(P16-P13))</f>
         <v>9</v>
       </c>
       <c r="Q17" s="9" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
     </row>
   </sheetData>
@@ -2291,18 +2450,18 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD44C968-61FF-4F4E-9D6C-A1C9337DEECD}">
-  <dimension ref="B1:Q8"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="35.25" customHeight="1" x14ac:dyDescent="0.3"/>
+  <dimension ref="B1:Q17"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="35.25" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="40.6640625" style="5" customWidth="1"/>
-    <col min="2" max="2" width="58.6640625" style="5" customWidth="1"/>
-    <col min="3" max="3" width="33.88671875" style="5" customWidth="1"/>
-    <col min="4" max="4" width="17.5546875" style="5" customWidth="1"/>
-    <col min="5" max="5" width="9.6640625" style="5" customWidth="1"/>
-    <col min="6" max="16384" width="9.109375" style="5"/>
+    <col min="1" max="1" width="40.7109375" style="5" customWidth="1"/>
+    <col min="2" max="2" width="58.7109375" style="5" customWidth="1"/>
+    <col min="3" max="3" width="68.85546875" style="5" customWidth="1"/>
+    <col min="4" max="4" width="17.5703125" style="5" customWidth="1"/>
+    <col min="5" max="5" width="9.7109375" style="5" customWidth="1"/>
+    <col min="6" max="16384" width="9.140625" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:17" ht="150" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:17" ht="150" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -2320,7 +2479,7 @@
       <c r="P1" s="1"/>
       <c r="Q1" s="1"/>
     </row>
-    <row r="2" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="10" t="s">
         <v>6</v>
       </c>
@@ -2346,34 +2505,34 @@
       <c r="P2" s="1"/>
       <c r="Q2" s="1"/>
     </row>
-    <row r="3" spans="2:17" ht="75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:17" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="1" t="s">
-        <v>92</v>
+        <v>136</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="D3" s="5">
-        <v>2.5</v>
+        <v>2.65</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="2:17" ht="75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:17" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
-        <v>94</v>
+        <v>137</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="D4" s="1">
-        <v>3.5</v>
+        <v>3.65</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="F4" s="1"/>
+      <c r="F4"/>
       <c r="G4" s="1"/>
       <c r="H4" s="10"/>
       <c r="I4" s="10"/>
@@ -2386,8 +2545,10 @@
       <c r="P4" s="10"/>
       <c r="Q4" s="10"/>
     </row>
-    <row r="5" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="1"/>
+    <row r="5" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="1" t="s">
+        <v>128</v>
+      </c>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
@@ -2404,7 +2565,7 @@
       <c r="P5" s="14"/>
       <c r="Q5" s="1"/>
     </row>
-    <row r="6" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="1"/>
       <c r="C6" s="9"/>
       <c r="D6" s="1"/>
@@ -2422,11 +2583,16 @@
       <c r="P6" s="14"/>
       <c r="Q6" s="1"/>
     </row>
-    <row r="7" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="1"/>
-      <c r="C7" s="1"/>
-      <c r="D7" s="1"/>
-      <c r="E7" s="6"/>
+    <row r="7" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="D7" s="5">
+        <v>560</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>36</v>
+      </c>
       <c r="F7" s="1"/>
       <c r="G7" s="1"/>
       <c r="H7" s="1"/>
@@ -2440,11 +2606,17 @@
       <c r="P7" s="1"/>
       <c r="Q7" s="1"/>
     </row>
-    <row r="8" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="1"/>
+    <row r="8" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="1" t="s">
+        <v>131</v>
+      </c>
       <c r="C8" s="1"/>
-      <c r="D8" s="1"/>
-      <c r="E8" s="1"/>
+      <c r="D8" s="1">
+        <v>1200</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>36</v>
+      </c>
       <c r="F8" s="1"/>
       <c r="G8" s="1"/>
       <c r="H8" s="1"/>
@@ -2458,7 +2630,89 @@
       <c r="P8" s="1"/>
       <c r="Q8" s="1"/>
     </row>
+    <row r="9" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="D9" s="1">
+        <f>5*D8/(D8+D7)</f>
+        <v>3.4090909090909092</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="11" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="D11" s="5">
+        <v>82</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="12" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="D12" s="5">
+        <v>33</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="13" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="D13" s="5">
+        <f>(1+D11/D12)*D3-D11/D12*D9</f>
+        <v>0.76377410468319518</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="D14" s="5">
+        <f>(1+D11/D12)*D4-D11/D12*D9</f>
+        <v>4.2486225895316796</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="15" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="32" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="16" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B16" s="32"/>
+    </row>
+    <row r="17" spans="2:6" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B17" s="32"/>
+      <c r="F17"/>
+    </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B15:B17"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -2466,15 +2720,15 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CBC3F59B-30C5-40B9-A90E-89A9AC3DA184}">
-  <dimension ref="A1:S17"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="35.25" customHeight="1" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:S22"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="35.25" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="40.6640625" style="5" customWidth="1"/>
-    <col min="2" max="20" width="16.6640625" style="5" customWidth="1"/>
-    <col min="21" max="16384" width="9.109375" style="5"/>
+    <col min="1" max="1" width="40.7109375" style="5" customWidth="1"/>
+    <col min="2" max="20" width="16.7109375" style="5" customWidth="1"/>
+    <col min="21" max="16384" width="9.140625" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="150" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:19" ht="150" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B1" s="15"/>
       <c r="C1" s="15"/>
       <c r="D1" s="15"/>
@@ -2494,134 +2748,134 @@
       <c r="R1" s="15"/>
       <c r="S1" s="15"/>
     </row>
-    <row r="2" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="28" t="s">
+    <row r="2" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2" s="30" t="s">
+        <v>68</v>
+      </c>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30" t="s">
+        <v>69</v>
+      </c>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30" t="s">
         <v>70</v>
       </c>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28" t="s">
+      <c r="G2" s="30"/>
+      <c r="H2" s="10"/>
+      <c r="I2" s="30" t="s">
+        <v>80</v>
+      </c>
+      <c r="J2" s="30"/>
+      <c r="K2" s="30"/>
+      <c r="L2" s="30"/>
+    </row>
+    <row r="3" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="C3" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="E2" s="28"/>
-      <c r="F2" s="28" t="s">
+      <c r="D3" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="F3" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="G3" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="I3" s="30" t="s">
+        <v>67</v>
+      </c>
+      <c r="J3" s="30"/>
+      <c r="K3" s="30" t="s">
+        <v>71</v>
+      </c>
+      <c r="L3" s="30"/>
+    </row>
+    <row r="4" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="G2" s="28"/>
-      <c r="H2" s="10"/>
-      <c r="I2" s="28" t="s">
-        <v>82</v>
-      </c>
-      <c r="J2" s="28"/>
-      <c r="K2" s="28"/>
-      <c r="L2" s="28"/>
-    </row>
-    <row r="3" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="10" t="s">
-        <v>69</v>
-      </c>
-      <c r="C3" s="10" t="s">
-        <v>73</v>
-      </c>
-      <c r="D3" s="10" t="s">
-        <v>69</v>
-      </c>
-      <c r="E3" s="10" t="s">
-        <v>73</v>
-      </c>
-      <c r="F3" s="10" t="s">
-        <v>69</v>
-      </c>
-      <c r="G3" s="10" t="s">
-        <v>73</v>
-      </c>
-      <c r="I3" s="28" t="s">
-        <v>69</v>
-      </c>
-      <c r="J3" s="28"/>
-      <c r="K3" s="28" t="s">
-        <v>73</v>
-      </c>
-      <c r="L3" s="28"/>
-    </row>
-    <row r="4" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
-        <v>74</v>
-      </c>
       <c r="B4" s="1">
-        <v>4.2</v>
+        <v>4.25</v>
       </c>
       <c r="C4" s="1">
-        <v>0.8</v>
+        <v>0.75</v>
       </c>
       <c r="D4" s="1">
-        <v>3.5</v>
+        <v>4.25</v>
       </c>
       <c r="E4" s="1">
-        <v>2.5</v>
+        <v>0.75</v>
       </c>
       <c r="F4" s="1">
-        <v>4.5</v>
+        <v>4.25</v>
       </c>
       <c r="G4" s="1">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="H4" s="10"/>
       <c r="I4" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="K4" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="J4" s="1" t="s">
+      <c r="L4" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="K4" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="L4" s="1" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="5" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="5" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B5" s="18">
         <f>5*C11/(B11+C11)</f>
-        <v>4.2572463768115938</v>
+        <v>4.25</v>
       </c>
       <c r="C5" s="18">
         <f>5*E11/(D11+E11)</f>
-        <v>0.74275362318840576</v>
+        <v>0.75</v>
       </c>
       <c r="D5" s="18">
         <f>5*G11/(F11+G11)</f>
-        <v>3.5652173913043477</v>
+        <v>4.25</v>
       </c>
       <c r="E5" s="18">
         <f>5*I11/(H11+I11)</f>
-        <v>2.5</v>
+        <v>0.75</v>
       </c>
       <c r="F5" s="18">
         <f>5*K11/(J11+K11)</f>
-        <v>4.4676806083650185</v>
+        <v>4.25</v>
       </c>
       <c r="G5" s="18">
         <f>5*M11/(L11+M11)</f>
-        <v>0.53231939163498099</v>
+        <v>0.75</v>
       </c>
       <c r="H5" s="1"/>
       <c r="I5" s="1" t="s">
         <v>50</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="K5" s="1" t="s">
         <v>50</v>
       </c>
       <c r="L5" s="1" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="6" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="1"/>
       <c r="C6" s="9"/>
       <c r="D6" s="1"/>
@@ -2639,7 +2893,7 @@
       <c r="R6" s="1"/>
       <c r="S6" s="1"/>
     </row>
-    <row r="7" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
@@ -2659,25 +2913,25 @@
       <c r="R7" s="1"/>
       <c r="S7" s="1"/>
     </row>
-    <row r="8" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="28" t="s">
+    <row r="8" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="30" t="s">
+        <v>68</v>
+      </c>
+      <c r="C8" s="30"/>
+      <c r="D8" s="30"/>
+      <c r="E8" s="30"/>
+      <c r="F8" s="30" t="s">
+        <v>69</v>
+      </c>
+      <c r="G8" s="30"/>
+      <c r="H8" s="30"/>
+      <c r="I8" s="30"/>
+      <c r="J8" s="30" t="s">
         <v>70</v>
       </c>
-      <c r="C8" s="28"/>
-      <c r="D8" s="28"/>
-      <c r="E8" s="28"/>
-      <c r="F8" s="28" t="s">
-        <v>71</v>
-      </c>
-      <c r="G8" s="28"/>
-      <c r="H8" s="28"/>
-      <c r="I8" s="28"/>
-      <c r="J8" s="28" t="s">
-        <v>72</v>
-      </c>
-      <c r="K8" s="28"/>
-      <c r="L8" s="28"/>
-      <c r="M8" s="28"/>
+      <c r="K8" s="30"/>
+      <c r="L8" s="30"/>
+      <c r="M8" s="30"/>
       <c r="N8" s="1"/>
       <c r="O8" s="1"/>
       <c r="P8" s="1"/>
@@ -2685,195 +2939,228 @@
       <c r="R8" s="1"/>
       <c r="S8" s="1"/>
     </row>
-    <row r="9" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="28" t="s">
-        <v>69</v>
-      </c>
-      <c r="C9" s="28"/>
-      <c r="D9" s="28" t="s">
-        <v>73</v>
-      </c>
-      <c r="E9" s="28"/>
-      <c r="F9" s="28" t="s">
-        <v>69</v>
-      </c>
-      <c r="G9" s="28"/>
-      <c r="H9" s="28" t="s">
-        <v>73</v>
-      </c>
-      <c r="I9" s="28"/>
-      <c r="J9" s="28" t="s">
-        <v>69</v>
-      </c>
-      <c r="K9" s="28"/>
-      <c r="L9" s="28" t="s">
-        <v>73</v>
-      </c>
-      <c r="M9" s="28"/>
-    </row>
-    <row r="10" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="30" t="s">
+        <v>67</v>
+      </c>
+      <c r="C9" s="30"/>
+      <c r="D9" s="30" t="s">
+        <v>71</v>
+      </c>
+      <c r="E9" s="30"/>
+      <c r="F9" s="30" t="s">
+        <v>67</v>
+      </c>
+      <c r="G9" s="30"/>
+      <c r="H9" s="30" t="s">
+        <v>71</v>
+      </c>
+      <c r="I9" s="30"/>
+      <c r="J9" s="30" t="s">
+        <v>67</v>
+      </c>
+      <c r="K9" s="30"/>
+      <c r="L9" s="30" t="s">
+        <v>71</v>
+      </c>
+      <c r="M9" s="30"/>
+    </row>
+    <row r="10" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="1" t="s">
         <v>56</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>56</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="F10" s="1" t="s">
         <v>56</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="H10" s="1" t="s">
         <v>56</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="J10" s="1" t="s">
         <v>56</v>
       </c>
       <c r="K10" s="1" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="L10" s="1" t="s">
         <v>56</v>
       </c>
       <c r="M10" s="1" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="11" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="11" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B11" s="17">
-        <v>8.1999999999999993</v>
+        <v>120</v>
       </c>
       <c r="C11" s="18">
-        <v>47</v>
+        <v>680</v>
       </c>
       <c r="D11" s="18">
-        <v>47</v>
+        <v>680</v>
       </c>
       <c r="E11" s="18">
-        <v>8.1999999999999993</v>
+        <v>120</v>
       </c>
       <c r="F11" s="17">
-        <v>3.3</v>
+        <v>120</v>
       </c>
       <c r="G11" s="18">
-        <v>8.1999999999999993</v>
+        <v>680</v>
       </c>
       <c r="H11" s="18">
-        <v>47</v>
+        <v>680</v>
       </c>
       <c r="I11" s="18">
-        <v>47</v>
+        <v>120</v>
       </c>
       <c r="J11" s="17">
-        <v>5.6</v>
+        <v>120</v>
       </c>
       <c r="K11" s="18">
-        <v>47</v>
+        <v>680</v>
       </c>
       <c r="L11" s="18">
-        <v>47</v>
+        <v>680</v>
       </c>
       <c r="M11" s="18">
-        <v>5.6</v>
+        <v>120</v>
       </c>
       <c r="N11" s="1" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="13" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C13" s="21" t="s">
+        <v>123</v>
+      </c>
+      <c r="D13" s="5">
+        <f>5/(B11+C11)</f>
+        <v>6.2500000000000003E-3</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="14" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C14" s="21" t="s">
+        <v>124</v>
+      </c>
+      <c r="D14" s="5">
+        <f>D13^2*C11</f>
+        <v>2.6562500000000006E-2</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F14" s="20" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="18" spans="2:8" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B18" s="30" t="s">
+        <v>68</v>
+      </c>
+      <c r="C18" s="30"/>
+      <c r="D18" s="30" t="s">
+        <v>69</v>
+      </c>
+      <c r="E18" s="30"/>
+      <c r="F18" s="30" t="s">
+        <v>70</v>
+      </c>
+      <c r="G18" s="30"/>
+    </row>
+    <row r="19" spans="2:8" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B19" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="F19" s="1" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="13" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="28" t="s">
-        <v>70</v>
-      </c>
-      <c r="C13" s="28"/>
-      <c r="D13" s="28" t="s">
-        <v>71</v>
-      </c>
-      <c r="E13" s="28"/>
-      <c r="F13" s="28" t="s">
-        <v>72</v>
-      </c>
-      <c r="G13" s="28"/>
-    </row>
-    <row r="14" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="1" t="s">
+      <c r="G19" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="C14" s="1" t="s">
+    </row>
+    <row r="20" spans="2:8" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="5">
+        <f>(C5-2.5)/(100*0.068)</f>
+        <v>-0.25735294117647056</v>
+      </c>
+      <c r="C20" s="5">
+        <f>(B5-2.5)/(100*0.068)</f>
+        <v>0.25735294117647056</v>
+      </c>
+      <c r="D20" s="19">
+        <f>(E5+'Voltage Sensor'!D11/'Voltage Sensor'!D12*'Voltage Sensor'!D9)/(1+'Voltage Sensor'!D11/'Voltage Sensor'!D12)</f>
+        <v>2.6460474308300395</v>
+      </c>
+      <c r="E20" s="19">
+        <f>(D5+'Voltage Sensor'!D11/'Voltage Sensor'!D12*'Voltage Sensor'!D9)/(1+'Voltage Sensor'!D11/'Voltage Sensor'!D12)</f>
+        <v>3.6503952569169962</v>
+      </c>
+      <c r="F20" s="5">
+        <f>10000*G5/(5-G5)</f>
+        <v>1764.7058823529412</v>
+      </c>
+      <c r="G20" s="5">
+        <f>10000*F5/(5-F5)</f>
+        <v>56666.666666666664</v>
+      </c>
+    </row>
+    <row r="21" spans="2:8" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F21" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="D14" s="1" t="s">
+      <c r="G21" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="E14" s="1" t="s">
+    </row>
+    <row r="22" spans="2:8" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F22" s="5">
+        <v>66.3</v>
+      </c>
+      <c r="G22" s="5">
+        <v>-8</v>
+      </c>
+      <c r="H22" s="20" t="s">
         <v>102</v>
-      </c>
-      <c r="F14" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="G14" s="1" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="15" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="5">
-        <f>(C5-2.5)/(100*0.068)</f>
-        <v>-0.25841858482523444</v>
-      </c>
-      <c r="C15" s="5">
-        <f>(B5-2.5)/(100*0.068)</f>
-        <v>0.25841858482523433</v>
-      </c>
-      <c r="D15" s="19">
-        <f>E5</f>
-        <v>2.5</v>
-      </c>
-      <c r="E15" s="19">
-        <f>D5</f>
-        <v>3.5652173913043477</v>
-      </c>
-      <c r="F15" s="5">
-        <f>10000*G5/(5-G5)</f>
-        <v>1191.4893617021276</v>
-      </c>
-      <c r="G15" s="5">
-        <f>10000*F5/(5-F5)</f>
-        <v>83928.571428571333</v>
-      </c>
-    </row>
-    <row r="16" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="F16" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="G16" s="1" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="17" spans="6:8" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="F17" s="5">
-        <v>77</v>
-      </c>
-      <c r="G17" s="5">
-        <v>-10.1</v>
-      </c>
-      <c r="H17" s="20" t="s">
-        <v>107</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="D18:E18"/>
+    <mergeCell ref="F18:G18"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:L2"/>
     <mergeCell ref="I3:J3"/>
     <mergeCell ref="K3:L3"/>
@@ -2886,12 +3173,6 @@
     <mergeCell ref="H9:I9"/>
     <mergeCell ref="J9:K9"/>
     <mergeCell ref="L9:M9"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="D13:E13"/>
-    <mergeCell ref="F13:G13"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="F2:G2"/>
   </mergeCells>
   <phoneticPr fontId="11" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2902,17 +3183,17 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2DDA2E54-9BDB-4BF6-80B7-49457B01E1DD}">
   <dimension ref="B1:Q11"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="35.25" customHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="35.25" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="40.6640625" style="5" customWidth="1"/>
-    <col min="2" max="2" width="34.44140625" style="5" customWidth="1"/>
-    <col min="3" max="3" width="52.88671875" style="5" customWidth="1"/>
-    <col min="4" max="4" width="17.5546875" style="5" customWidth="1"/>
-    <col min="5" max="5" width="9.6640625" style="5" customWidth="1"/>
-    <col min="6" max="16384" width="9.109375" style="5"/>
+    <col min="1" max="1" width="40.7109375" style="5" customWidth="1"/>
+    <col min="2" max="2" width="34.42578125" style="5" customWidth="1"/>
+    <col min="3" max="3" width="52.85546875" style="5" customWidth="1"/>
+    <col min="4" max="4" width="17.5703125" style="5" customWidth="1"/>
+    <col min="5" max="5" width="9.7109375" style="5" customWidth="1"/>
+    <col min="6" max="16384" width="9.140625" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:17" ht="150" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:17" ht="150" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -2930,7 +3211,7 @@
       <c r="P1" s="1"/>
       <c r="Q1" s="1"/>
     </row>
-    <row r="2" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="10" t="s">
         <v>6</v>
       </c>
@@ -2956,33 +3237,33 @@
       <c r="P2" s="1"/>
       <c r="Q2" s="1"/>
     </row>
-    <row r="3" spans="2:17" ht="73.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:17" ht="73.900000000000006" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C3" s="9" t="s">
         <v>85</v>
-      </c>
-      <c r="C3" s="9" t="s">
-        <v>87</v>
       </c>
       <c r="D3" s="5">
         <v>16000</v>
       </c>
       <c r="E3" s="1" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="4" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="1" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="4" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="1" t="s">
-        <v>88</v>
-      </c>
       <c r="C4" s="1" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D4" s="5">
         <f>D3 / 2</f>
         <v>8000</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
@@ -2997,7 +3278,7 @@
       <c r="P4" s="10"/>
       <c r="Q4" s="10"/>
     </row>
-    <row r="5" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="1" t="s">
         <v>56</v>
       </c>
@@ -3023,19 +3304,19 @@
       <c r="P5" s="14"/>
       <c r="Q5" s="1"/>
     </row>
-    <row r="6" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="1" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D6" s="1">
         <f>1 / (2 * PI() * D5 *D4)</f>
         <v>4.232844231167429E-9</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="F6" s="1"/>
       <c r="G6" s="1"/>
@@ -3050,7 +3331,7 @@
       <c r="P6" s="14"/>
       <c r="Q6" s="1"/>
     </row>
-    <row r="7" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
@@ -3068,9 +3349,9 @@
       <c r="P7" s="1"/>
       <c r="Q7" s="1"/>
     </row>
-    <row r="8" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="10" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="C8" s="10" t="s">
         <v>7</v>
@@ -3094,7 +3375,7 @@
       <c r="P8" s="1"/>
       <c r="Q8" s="1"/>
     </row>
-    <row r="9" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="1" t="s">
         <v>56</v>
       </c>
@@ -3105,31 +3386,31 @@
         <v>36</v>
       </c>
     </row>
-    <row r="10" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="1" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="D10" s="5">
         <f>0.0000000047</f>
         <v>4.6999999999999999E-9</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="11" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="11" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="1" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="D11" s="5">
         <f>1/(2*PI()*D9*D10)</f>
         <v>7204.8412445403055</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
   </sheetData>
@@ -3143,17 +3424,17 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDBF5C97-B701-49E8-8D17-B57E480030E6}">
   <dimension ref="B1:Q15"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="35.25" customHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="35.25" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="40.6640625" style="5" customWidth="1"/>
-    <col min="2" max="2" width="34.44140625" style="5" customWidth="1"/>
-    <col min="3" max="3" width="52.88671875" style="5" customWidth="1"/>
-    <col min="4" max="4" width="17.5546875" style="5" customWidth="1"/>
-    <col min="5" max="5" width="9.6640625" style="5" customWidth="1"/>
-    <col min="6" max="16384" width="9.109375" style="5"/>
+    <col min="1" max="1" width="40.7109375" style="5" customWidth="1"/>
+    <col min="2" max="2" width="34.42578125" style="5" customWidth="1"/>
+    <col min="3" max="3" width="52.85546875" style="5" customWidth="1"/>
+    <col min="4" max="4" width="17.5703125" style="5" customWidth="1"/>
+    <col min="5" max="5" width="9.7109375" style="5" customWidth="1"/>
+    <col min="6" max="16384" width="9.140625" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:17" ht="150" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:17" ht="150" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -3171,7 +3452,7 @@
       <c r="P1" s="1"/>
       <c r="Q1" s="1"/>
     </row>
-    <row r="2" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="10" t="s">
         <v>6</v>
       </c>
@@ -3197,7 +3478,7 @@
       <c r="P2" s="1"/>
       <c r="Q2" s="1"/>
     </row>
-    <row r="3" spans="2:17" ht="73.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:17" ht="73.900000000000006" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="1" t="s">
         <v>56</v>
       </c>
@@ -3209,9 +3490,9 @@
         <v>36</v>
       </c>
     </row>
-    <row r="4" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C4" s="1"/>
       <c r="D4" s="1">
@@ -3233,9 +3514,9 @@
       <c r="P4" s="10"/>
       <c r="Q4" s="10"/>
     </row>
-    <row r="5" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C5" s="1"/>
       <c r="D5" s="16">
@@ -3257,7 +3538,7 @@
       <c r="P5" s="14"/>
       <c r="Q5" s="1"/>
     </row>
-    <row r="6" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="1" t="s">
         <v>30</v>
       </c>
@@ -3281,18 +3562,18 @@
       <c r="P6" s="14"/>
       <c r="Q6" s="1"/>
     </row>
-    <row r="7" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="21" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="D7" s="16">
         <v>1E-10</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="F7" s="1"/>
       <c r="G7" s="1"/>
@@ -3307,19 +3588,19 @@
       <c r="P7" s="1"/>
       <c r="Q7" s="1"/>
     </row>
-    <row r="8" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="21" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="D8" s="16">
         <f>D7*1.05</f>
         <v>1.0500000000000001E-10</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="F8" s="1"/>
       <c r="G8" s="1"/>
@@ -3334,68 +3615,68 @@
       <c r="P8" s="1"/>
       <c r="Q8" s="1"/>
     </row>
-    <row r="10" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="1" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="D10" s="22">
         <f>1/(-2*LN(1/3)*D5*D7)</f>
         <v>9683.3960279450785</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="11" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="11" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="1" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="D11" s="22">
         <f>1/(-2*LN(1/3)*D5*D8)</f>
         <v>9222.2819313762629</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="13" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="13" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="1" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="D13" s="16">
         <v>2000000</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="14" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="14" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="21" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="D14" s="23">
         <f>D13/D10</f>
         <v>206.53911026960463</v>
       </c>
     </row>
-    <row r="15" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="21" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="D15" s="23">
         <f>D13/D11</f>

</xml_diff>

<commit_message>
Added temperature lookup table to smarts excel
</commit_message>
<xml_diff>
--- a/Excel/sensors.xlsx
+++ b/Excel/sensors.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d393d29289b0eecc/Documents/School Stuff/ELECTENG 311/311/Excel/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uoa-my.sharepoint.com/personal/ctra157_uoa_auckland_ac_nz/Documents/Documents/GitHub/311/Excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="135" documentId="13_ncr:1_{FEF83167-29AA-4D2C-9F19-8FB03B27FB56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{12279AB5-856C-4769-9720-6B7ED887E860}"/>
+  <xr:revisionPtr revIDLastSave="208" documentId="13_ncr:1_{FEF83167-29AA-4D2C-9F19-8FB03B27FB56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{89A6A94C-C3E5-4D4D-B720-7A07230B4FEB}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="649" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Current Sensor" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,7 @@
     <sheet name="Window Comparator" sheetId="6" r:id="rId4"/>
     <sheet name="Anti-Aliasing Filter" sheetId="9" r:id="rId5"/>
     <sheet name="Touch Sensor Oscillator" sheetId="11" r:id="rId6"/>
+    <sheet name="Temp Sensor Lookup Table" sheetId="12" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -136,7 +137,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="147">
   <si>
     <t>Current Sense Amplifier</t>
   </si>
@@ -606,6 +607,18 @@
   <si>
     <t>Note: output calculations assume amplifier circuit has negligible loading on the voltage reference divider.</t>
   </si>
+  <si>
+    <t>Temperature (°C)</t>
+  </si>
+  <si>
+    <t>Resistance (Ω)</t>
+  </si>
+  <si>
+    <t>Output voltage (V)</t>
+  </si>
+  <si>
+    <t>Grey resistance cells are linearly interpolated from adjacent resistances given in datasheet.</t>
+  </si>
 </sst>
 </file>
 
@@ -615,7 +628,7 @@
     <numFmt numFmtId="164" formatCode="0.000000"/>
     <numFmt numFmtId="165" formatCode="0.000E+00"/>
     <numFmt numFmtId="166" formatCode="0.000"/>
-    <numFmt numFmtId="169" formatCode="0.0000E+00"/>
+    <numFmt numFmtId="167" formatCode="0.0000E+00"/>
   </numFmts>
   <fonts count="17" x14ac:knownFonts="1">
     <font>
@@ -738,7 +751,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -748,6 +761,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -764,7 +783,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -838,8 +857,11 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -854,14 +876,13 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1709,24 +1730,24 @@
       <c r="K3" s="1"/>
     </row>
     <row r="4" spans="2:17" ht="73.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="26"/>
-      <c r="C4" s="26"/>
-      <c r="D4" s="26"/>
-      <c r="E4" s="26"/>
+      <c r="B4" s="27"/>
+      <c r="C4" s="27"/>
+      <c r="D4" s="27"/>
+      <c r="E4" s="27"/>
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
-      <c r="H4" s="28" t="s">
+      <c r="H4" s="29" t="s">
         <v>4</v>
       </c>
-      <c r="I4" s="29"/>
-      <c r="J4" s="29"/>
-      <c r="K4" s="29"/>
-      <c r="N4" s="27" t="s">
+      <c r="I4" s="30"/>
+      <c r="J4" s="30"/>
+      <c r="K4" s="30"/>
+      <c r="N4" s="28" t="s">
         <v>5</v>
       </c>
-      <c r="O4" s="27"/>
-      <c r="P4" s="27"/>
-      <c r="Q4" s="27"/>
+      <c r="O4" s="28"/>
+      <c r="P4" s="28"/>
+      <c r="Q4" s="28"/>
     </row>
     <row r="5" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="10" t="s">
@@ -2190,7 +2211,7 @@
       <c r="O5" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="P5" s="31">
+      <c r="P5" s="25">
         <f>POWER(J7,2)*(D5+D7)</f>
         <v>3.3903900917282403E-4</v>
       </c>
@@ -2234,7 +2255,7 @@
       <c r="O6" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="P6" s="31">
+      <c r="P6" s="25">
         <f>POWER(J8, 2) * (D6+D8)</f>
         <v>2.1128605596545053E-3</v>
       </c>
@@ -2349,12 +2370,12 @@
       <c r="Q10" s="10"/>
     </row>
     <row r="11" spans="2:17" ht="99.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="N11" s="25" t="s">
+      <c r="N11" s="31" t="s">
         <v>121</v>
       </c>
-      <c r="O11" s="25"/>
-      <c r="P11" s="25"/>
-      <c r="Q11" s="25"/>
+      <c r="O11" s="31"/>
+      <c r="P11" s="31"/>
+      <c r="Q11" s="31"/>
     </row>
     <row r="12" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="N12" s="10" t="s">
@@ -2749,25 +2770,25 @@
       <c r="S1" s="15"/>
     </row>
     <row r="2" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="30" t="s">
+      <c r="B2" s="26" t="s">
         <v>68</v>
       </c>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30" t="s">
+      <c r="C2" s="26"/>
+      <c r="D2" s="26" t="s">
         <v>69</v>
       </c>
-      <c r="E2" s="30"/>
-      <c r="F2" s="30" t="s">
+      <c r="E2" s="26"/>
+      <c r="F2" s="26" t="s">
         <v>70</v>
       </c>
-      <c r="G2" s="30"/>
+      <c r="G2" s="26"/>
       <c r="H2" s="10"/>
-      <c r="I2" s="30" t="s">
+      <c r="I2" s="26" t="s">
         <v>80</v>
       </c>
-      <c r="J2" s="30"/>
-      <c r="K2" s="30"/>
-      <c r="L2" s="30"/>
+      <c r="J2" s="26"/>
+      <c r="K2" s="26"/>
+      <c r="L2" s="26"/>
     </row>
     <row r="3" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="10" t="s">
@@ -2788,14 +2809,14 @@
       <c r="G3" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="I3" s="30" t="s">
+      <c r="I3" s="26" t="s">
         <v>67</v>
       </c>
-      <c r="J3" s="30"/>
-      <c r="K3" s="30" t="s">
+      <c r="J3" s="26"/>
+      <c r="K3" s="26" t="s">
         <v>71</v>
       </c>
-      <c r="L3" s="30"/>
+      <c r="L3" s="26"/>
     </row>
     <row r="4" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
@@ -2914,24 +2935,24 @@
       <c r="S7" s="1"/>
     </row>
     <row r="8" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="30" t="s">
+      <c r="B8" s="26" t="s">
         <v>68</v>
       </c>
-      <c r="C8" s="30"/>
-      <c r="D8" s="30"/>
-      <c r="E8" s="30"/>
-      <c r="F8" s="30" t="s">
+      <c r="C8" s="26"/>
+      <c r="D8" s="26"/>
+      <c r="E8" s="26"/>
+      <c r="F8" s="26" t="s">
         <v>69</v>
       </c>
-      <c r="G8" s="30"/>
-      <c r="H8" s="30"/>
-      <c r="I8" s="30"/>
-      <c r="J8" s="30" t="s">
+      <c r="G8" s="26"/>
+      <c r="H8" s="26"/>
+      <c r="I8" s="26"/>
+      <c r="J8" s="26" t="s">
         <v>70</v>
       </c>
-      <c r="K8" s="30"/>
-      <c r="L8" s="30"/>
-      <c r="M8" s="30"/>
+      <c r="K8" s="26"/>
+      <c r="L8" s="26"/>
+      <c r="M8" s="26"/>
       <c r="N8" s="1"/>
       <c r="O8" s="1"/>
       <c r="P8" s="1"/>
@@ -2940,30 +2961,30 @@
       <c r="S8" s="1"/>
     </row>
     <row r="9" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="30" t="s">
+      <c r="B9" s="26" t="s">
         <v>67</v>
       </c>
-      <c r="C9" s="30"/>
-      <c r="D9" s="30" t="s">
+      <c r="C9" s="26"/>
+      <c r="D9" s="26" t="s">
         <v>71</v>
       </c>
-      <c r="E9" s="30"/>
-      <c r="F9" s="30" t="s">
+      <c r="E9" s="26"/>
+      <c r="F9" s="26" t="s">
         <v>67</v>
       </c>
-      <c r="G9" s="30"/>
-      <c r="H9" s="30" t="s">
+      <c r="G9" s="26"/>
+      <c r="H9" s="26" t="s">
         <v>71</v>
       </c>
-      <c r="I9" s="30"/>
-      <c r="J9" s="30" t="s">
+      <c r="I9" s="26"/>
+      <c r="J9" s="26" t="s">
         <v>67</v>
       </c>
-      <c r="K9" s="30"/>
-      <c r="L9" s="30" t="s">
+      <c r="K9" s="26"/>
+      <c r="L9" s="26" t="s">
         <v>71</v>
       </c>
-      <c r="M9" s="30"/>
+      <c r="M9" s="26"/>
     </row>
     <row r="10" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="1" t="s">
@@ -3075,18 +3096,18 @@
       </c>
     </row>
     <row r="18" spans="2:8" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="30" t="s">
+      <c r="B18" s="26" t="s">
         <v>68</v>
       </c>
-      <c r="C18" s="30"/>
-      <c r="D18" s="30" t="s">
+      <c r="C18" s="26"/>
+      <c r="D18" s="26" t="s">
         <v>69</v>
       </c>
-      <c r="E18" s="30"/>
-      <c r="F18" s="30" t="s">
+      <c r="E18" s="26"/>
+      <c r="F18" s="26" t="s">
         <v>70</v>
       </c>
-      <c r="G18" s="30"/>
+      <c r="G18" s="26"/>
     </row>
     <row r="19" spans="2:8" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="1" t="s">
@@ -3155,12 +3176,6 @@
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="D18:E18"/>
-    <mergeCell ref="F18:G18"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:L2"/>
     <mergeCell ref="I3:J3"/>
     <mergeCell ref="K3:L3"/>
@@ -3173,6 +3188,12 @@
     <mergeCell ref="H9:I9"/>
     <mergeCell ref="J9:K9"/>
     <mergeCell ref="L9:M9"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="D18:E18"/>
+    <mergeCell ref="F18:G18"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="F2:G2"/>
   </mergeCells>
   <phoneticPr fontId="11" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3691,6 +3712,1416 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A1B340A-C562-401C-9C12-DAC3640D6A6E}">
+  <dimension ref="A1:F82"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="18.28515625" customWidth="1"/>
+    <col min="2" max="2" width="14.5703125" customWidth="1"/>
+    <col min="3" max="3" width="18.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>143</v>
+      </c>
+      <c r="B1" t="s">
+        <v>144</v>
+      </c>
+      <c r="C1" t="s">
+        <v>145</v>
+      </c>
+      <c r="D1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>-10</v>
+      </c>
+      <c r="B2">
+        <f>6.2927*10000</f>
+        <v>62927</v>
+      </c>
+      <c r="C2">
+        <f>B2/(B2+10000)*5</f>
+        <v>4.3143828760267118</v>
+      </c>
+      <c r="D2" s="34">
+        <f>C2*1000</f>
+        <v>4314.3828760267115</v>
+      </c>
+      <c r="F2" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>-9</v>
+      </c>
+      <c r="B3" s="33">
+        <f>4/5*B2+1/5*B7</f>
+        <v>59757.000000000007</v>
+      </c>
+      <c r="C3">
+        <f t="shared" ref="C3:C66" si="0">B3/(B3+10000)*5</f>
+        <v>4.2832260561664066</v>
+      </c>
+      <c r="D3" s="34">
+        <f t="shared" ref="D3:D66" si="1">C3*1000</f>
+        <v>4283.226056166407</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>-8</v>
+      </c>
+      <c r="B4" s="33">
+        <f>3/5*B2+2/5*B7</f>
+        <v>56587</v>
+      </c>
+      <c r="C4">
+        <f t="shared" si="0"/>
+        <v>4.2491026776998515</v>
+      </c>
+      <c r="D4" s="34">
+        <f t="shared" si="1"/>
+        <v>4249.1026776998515</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>-7</v>
+      </c>
+      <c r="B5" s="33">
+        <f>2/5*B2+3/5*B7</f>
+        <v>53417</v>
+      </c>
+      <c r="C5">
+        <f t="shared" si="0"/>
+        <v>4.2115678761215447</v>
+      </c>
+      <c r="D5" s="34">
+        <f t="shared" si="1"/>
+        <v>4211.5678761215449</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>-6</v>
+      </c>
+      <c r="B6" s="33">
+        <f>1/5*B2+4/5*B7</f>
+        <v>50247</v>
+      </c>
+      <c r="C6">
+        <f t="shared" si="0"/>
+        <v>4.1700831576676016</v>
+      </c>
+      <c r="D6" s="34">
+        <f t="shared" si="1"/>
+        <v>4170.0831576676019</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>-5</v>
+      </c>
+      <c r="B7">
+        <f>4.7077*10000</f>
+        <v>47077</v>
+      </c>
+      <c r="C7">
+        <f t="shared" si="0"/>
+        <v>4.1239903989347724</v>
+      </c>
+      <c r="D7" s="34">
+        <f t="shared" si="1"/>
+        <v>4123.9903989347722</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>-4</v>
+      </c>
+      <c r="B8" s="33">
+        <f>4/5*B7+1/5*B12</f>
+        <v>44774.2</v>
+      </c>
+      <c r="C8">
+        <f t="shared" si="0"/>
+        <v>4.0871614738325706</v>
+      </c>
+      <c r="D8" s="34">
+        <f t="shared" si="1"/>
+        <v>4087.1614738325707</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>-3</v>
+      </c>
+      <c r="B9" s="33">
+        <f>3/5*B7+2/5*B12</f>
+        <v>42471.4</v>
+      </c>
+      <c r="C9">
+        <f t="shared" si="0"/>
+        <v>4.0470999439694761</v>
+      </c>
+      <c r="D9" s="34">
+        <f t="shared" si="1"/>
+        <v>4047.099943969476</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>-2</v>
+      </c>
+      <c r="B10" s="33">
+        <f>2/5*B7+3/5*B12</f>
+        <v>40168.6</v>
+      </c>
+      <c r="C10">
+        <f t="shared" si="0"/>
+        <v>4.0033606678280833</v>
+      </c>
+      <c r="D10" s="34">
+        <f t="shared" si="1"/>
+        <v>4003.3606678280835</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>-1</v>
+      </c>
+      <c r="B11" s="33">
+        <f>1/5*B7+4/5*B12</f>
+        <v>37865.800000000003</v>
+      </c>
+      <c r="C11">
+        <f t="shared" si="0"/>
+        <v>3.9554128417366892</v>
+      </c>
+      <c r="D11" s="34">
+        <f t="shared" si="1"/>
+        <v>3955.4128417366892</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>0</v>
+      </c>
+      <c r="B12">
+        <f>3.5563*10000</f>
+        <v>35563</v>
+      </c>
+      <c r="C12">
+        <f t="shared" si="0"/>
+        <v>3.9026183526106712</v>
+      </c>
+      <c r="D12" s="34">
+        <f t="shared" si="1"/>
+        <v>3902.6183526106711</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>1</v>
+      </c>
+      <c r="B13" s="33">
+        <f>4/5*B12+1/5*B17</f>
+        <v>33874.200000000004</v>
+      </c>
+      <c r="C13">
+        <f t="shared" si="0"/>
+        <v>3.8603780809678585</v>
+      </c>
+      <c r="D13" s="34">
+        <f t="shared" si="1"/>
+        <v>3860.3780809678583</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>2</v>
+      </c>
+      <c r="B14" s="33">
+        <f>3/5*B12+2/5*B17</f>
+        <v>32185.4</v>
+      </c>
+      <c r="C14">
+        <f t="shared" si="0"/>
+        <v>3.8147558159932111</v>
+      </c>
+      <c r="D14" s="34">
+        <f t="shared" si="1"/>
+        <v>3814.7558159932109</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>3</v>
+      </c>
+      <c r="B15" s="33">
+        <f>2/5*B12+3/5*B17</f>
+        <v>30496.6</v>
+      </c>
+      <c r="C15">
+        <f t="shared" si="0"/>
+        <v>3.7653284473264419</v>
+      </c>
+      <c r="D15" s="34">
+        <f t="shared" si="1"/>
+        <v>3765.3284473264421</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>4</v>
+      </c>
+      <c r="B16" s="33">
+        <f>1/5*B12+4/5*B17</f>
+        <v>28807.800000000003</v>
+      </c>
+      <c r="C16">
+        <f t="shared" si="0"/>
+        <v>3.7115992145908812</v>
+      </c>
+      <c r="D16" s="34">
+        <f t="shared" si="1"/>
+        <v>3711.5992145908813</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>5</v>
+      </c>
+      <c r="B17">
+        <f>2.7119*10000</f>
+        <v>27119</v>
+      </c>
+      <c r="C17">
+        <f t="shared" si="0"/>
+        <v>3.6529809531506774</v>
+      </c>
+      <c r="D17" s="34">
+        <f t="shared" si="1"/>
+        <v>3652.9809531506776</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>6</v>
+      </c>
+      <c r="B18" s="33">
+        <f>4/5*B17+1/5*B22</f>
+        <v>25867.200000000001</v>
+      </c>
+      <c r="C18">
+        <f t="shared" si="0"/>
+        <v>3.6059686844805281</v>
+      </c>
+      <c r="D18" s="34">
+        <f t="shared" si="1"/>
+        <v>3605.9686844805283</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>7</v>
+      </c>
+      <c r="B19" s="33">
+        <f>3/5*B17+2/5*B22</f>
+        <v>24615.4</v>
+      </c>
+      <c r="C19">
+        <f t="shared" si="0"/>
+        <v>3.5555561975305787</v>
+      </c>
+      <c r="D19" s="34">
+        <f t="shared" si="1"/>
+        <v>3555.5561975305786</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>8</v>
+      </c>
+      <c r="B20" s="33">
+        <f>2/5*B17+3/5*B22</f>
+        <v>23363.599999999999</v>
+      </c>
+      <c r="C20">
+        <f t="shared" si="0"/>
+        <v>3.5013607644259008</v>
+      </c>
+      <c r="D20" s="34">
+        <f t="shared" si="1"/>
+        <v>3501.3607644259009</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>9</v>
+      </c>
+      <c r="B21" s="33">
+        <f>1/5*B17+4/5*B22</f>
+        <v>22111.8</v>
+      </c>
+      <c r="C21">
+        <f t="shared" si="0"/>
+        <v>3.4429399784502897</v>
+      </c>
+      <c r="D21" s="34">
+        <f t="shared" si="1"/>
+        <v>3442.9399784502898</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>10</v>
+      </c>
+      <c r="B22">
+        <f>2.086*10000</f>
+        <v>20860</v>
+      </c>
+      <c r="C22">
+        <f t="shared" si="0"/>
+        <v>3.3797796500324044</v>
+      </c>
+      <c r="D22" s="34">
+        <f t="shared" si="1"/>
+        <v>3379.7796500324043</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>11</v>
+      </c>
+      <c r="B23" s="33">
+        <f>4/5*B22+1/5*B27</f>
+        <v>19928.8</v>
+      </c>
+      <c r="C23">
+        <f t="shared" si="0"/>
+        <v>3.3293683675924193</v>
+      </c>
+      <c r="D23" s="34">
+        <f t="shared" si="1"/>
+        <v>3329.3683675924194</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>12</v>
+      </c>
+      <c r="B24" s="33">
+        <f>3/5*B22+2/5*B27</f>
+        <v>18997.599999999999</v>
+      </c>
+      <c r="C24">
+        <f t="shared" si="0"/>
+        <v>3.2757193698788867</v>
+      </c>
+      <c r="D24" s="34">
+        <f t="shared" si="1"/>
+        <v>3275.7193698788865</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>13</v>
+      </c>
+      <c r="B25" s="33">
+        <f>2/5*B22+3/5*B27</f>
+        <v>18066.400000000001</v>
+      </c>
+      <c r="C25">
+        <f t="shared" si="0"/>
+        <v>3.2185103896474079</v>
+      </c>
+      <c r="D25" s="34">
+        <f t="shared" si="1"/>
+        <v>3218.5103896474079</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>14</v>
+      </c>
+      <c r="B26" s="33">
+        <f>1/5*B22+4/5*B27</f>
+        <v>17135.2</v>
+      </c>
+      <c r="C26">
+        <f t="shared" si="0"/>
+        <v>3.1573749226097467</v>
+      </c>
+      <c r="D26" s="34">
+        <f t="shared" si="1"/>
+        <v>3157.3749226097466</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>15</v>
+      </c>
+      <c r="B27">
+        <f>1.6204*10000</f>
+        <v>16204</v>
+      </c>
+      <c r="C27">
+        <f t="shared" si="0"/>
+        <v>3.0918943672721722</v>
+      </c>
+      <c r="D27" s="34">
+        <f t="shared" si="1"/>
+        <v>3091.8943672721721</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>16</v>
+      </c>
+      <c r="B28" s="33">
+        <f>4/5*B27+1/5*B32</f>
+        <v>15499.800000000001</v>
+      </c>
+      <c r="C28">
+        <f t="shared" si="0"/>
+        <v>3.0392003074533918</v>
+      </c>
+      <c r="D28" s="34">
+        <f t="shared" si="1"/>
+        <v>3039.2003074533918</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>17</v>
+      </c>
+      <c r="B29" s="33">
+        <f>3/5*B27+2/5*B32</f>
+        <v>14795.6</v>
+      </c>
+      <c r="C29">
+        <f t="shared" si="0"/>
+        <v>2.9835132039555408</v>
+      </c>
+      <c r="D29" s="34">
+        <f t="shared" si="1"/>
+        <v>2983.5132039555406</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>18</v>
+      </c>
+      <c r="B30" s="33">
+        <f>2/5*B27+3/5*B32</f>
+        <v>14091.4</v>
+      </c>
+      <c r="C30">
+        <f t="shared" si="0"/>
+        <v>2.9245705936558268</v>
+      </c>
+      <c r="D30" s="34">
+        <f t="shared" si="1"/>
+        <v>2924.570593655827</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31">
+        <v>19</v>
+      </c>
+      <c r="B31" s="33">
+        <f>1/5*B27+4/5*B32</f>
+        <v>13387.2</v>
+      </c>
+      <c r="C31">
+        <f t="shared" si="0"/>
+        <v>2.8620784018608472</v>
+      </c>
+      <c r="D31" s="34">
+        <f t="shared" si="1"/>
+        <v>2862.078401860847</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32">
+        <v>20</v>
+      </c>
+      <c r="B32">
+        <f>1.2683*10000</f>
+        <v>12683</v>
+      </c>
+      <c r="C32">
+        <f t="shared" si="0"/>
+        <v>2.7957060353568752</v>
+      </c>
+      <c r="D32" s="34">
+        <f t="shared" si="1"/>
+        <v>2795.7060353568754</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A33">
+        <v>21</v>
+      </c>
+      <c r="B33" s="33">
+        <f>4/5*B32+1/5*B37</f>
+        <v>12146.400000000001</v>
+      </c>
+      <c r="C33">
+        <f t="shared" si="0"/>
+        <v>2.7422967163963445</v>
+      </c>
+      <c r="D33" s="34">
+        <f t="shared" si="1"/>
+        <v>2742.2967163963444</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A34">
+        <v>22</v>
+      </c>
+      <c r="B34" s="33">
+        <f>3/5*B32+2/5*B37</f>
+        <v>11609.8</v>
+      </c>
+      <c r="C34">
+        <f t="shared" si="0"/>
+        <v>2.6862349489583432</v>
+      </c>
+      <c r="D34" s="34">
+        <f t="shared" si="1"/>
+        <v>2686.2349489583435</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A35">
+        <v>23</v>
+      </c>
+      <c r="B35" s="33">
+        <f>2/5*B32+3/5*B37</f>
+        <v>11073.2</v>
+      </c>
+      <c r="C35">
+        <f t="shared" si="0"/>
+        <v>2.6273181102063288</v>
+      </c>
+      <c r="D35" s="34">
+        <f t="shared" si="1"/>
+        <v>2627.3181102063286</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36">
+        <v>24</v>
+      </c>
+      <c r="B36" s="33">
+        <f>1/5*B32+4/5*B37</f>
+        <v>10536.6</v>
+      </c>
+      <c r="C36">
+        <f t="shared" si="0"/>
+        <v>2.5653224000077914</v>
+      </c>
+      <c r="D36" s="34">
+        <f t="shared" si="1"/>
+        <v>2565.3224000077917</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A37">
+        <v>25</v>
+      </c>
+      <c r="B37">
+        <f>10000</f>
+        <v>10000</v>
+      </c>
+      <c r="C37">
+        <f t="shared" si="0"/>
+        <v>2.5</v>
+      </c>
+      <c r="D37" s="34">
+        <f t="shared" si="1"/>
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A38">
+        <v>26</v>
+      </c>
+      <c r="B38" s="33">
+        <f>4/5*B37+1/5*B42</f>
+        <v>9588.4</v>
+      </c>
+      <c r="C38">
+        <f t="shared" si="0"/>
+        <v>2.4474689101713256</v>
+      </c>
+      <c r="D38" s="34">
+        <f t="shared" si="1"/>
+        <v>2447.4689101713257</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A39">
+        <v>27</v>
+      </c>
+      <c r="B39" s="33">
+        <f>3/5*B37+2/5*B42</f>
+        <v>9176.7999999999993</v>
+      </c>
+      <c r="C39">
+        <f t="shared" si="0"/>
+        <v>2.3926828250803052</v>
+      </c>
+      <c r="D39" s="34">
+        <f t="shared" si="1"/>
+        <v>2392.6828250803051</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A40">
+        <v>28</v>
+      </c>
+      <c r="B40" s="33">
+        <f>2/5*B37+3/5*B42</f>
+        <v>8765.2000000000007</v>
+      </c>
+      <c r="C40">
+        <f t="shared" si="0"/>
+        <v>2.3354933600494534</v>
+      </c>
+      <c r="D40" s="34">
+        <f t="shared" si="1"/>
+        <v>2335.4933600494533</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A41">
+        <v>29</v>
+      </c>
+      <c r="B41" s="33">
+        <f>1/5*B37+4/5*B42</f>
+        <v>8353.6</v>
+      </c>
+      <c r="C41">
+        <f t="shared" si="0"/>
+        <v>2.275738819632116</v>
+      </c>
+      <c r="D41" s="34">
+        <f t="shared" si="1"/>
+        <v>2275.7388196321158</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A42">
+        <v>30</v>
+      </c>
+      <c r="B42">
+        <f>0.7942*10000</f>
+        <v>7942</v>
+      </c>
+      <c r="C42">
+        <f t="shared" si="0"/>
+        <v>2.2132426708282242</v>
+      </c>
+      <c r="D42" s="34">
+        <f t="shared" si="1"/>
+        <v>2213.2426708282242</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A43">
+        <v>31</v>
+      </c>
+      <c r="B43" s="33">
+        <f>4/5*B42+1/5*B47</f>
+        <v>7618.9600000000009</v>
+      </c>
+      <c r="C43">
+        <f t="shared" si="0"/>
+        <v>2.1621480496011118</v>
+      </c>
+      <c r="D43" s="34">
+        <f t="shared" si="1"/>
+        <v>2162.1480496011118</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A44">
+        <v>32</v>
+      </c>
+      <c r="B44" s="33">
+        <f>3/5*B42+2/5*B47</f>
+        <v>7295.92</v>
+      </c>
+      <c r="C44">
+        <f t="shared" si="0"/>
+        <v>2.1091448156559469</v>
+      </c>
+      <c r="D44" s="34">
+        <f t="shared" si="1"/>
+        <v>2109.1448156559468</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A45">
+        <v>33</v>
+      </c>
+      <c r="B45" s="33">
+        <f>2/5*B42+3/5*B47</f>
+        <v>6972.88</v>
+      </c>
+      <c r="C45">
+        <f t="shared" si="0"/>
+        <v>2.054123990742879</v>
+      </c>
+      <c r="D45" s="34">
+        <f t="shared" si="1"/>
+        <v>2054.123990742879</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A46">
+        <v>34</v>
+      </c>
+      <c r="B46" s="33">
+        <f>1/5*B42+4/5*B47</f>
+        <v>6649.84</v>
+      </c>
+      <c r="C46">
+        <f t="shared" si="0"/>
+        <v>1.9969681390331679</v>
+      </c>
+      <c r="D46" s="34">
+        <f t="shared" si="1"/>
+        <v>1996.968139033168</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A47">
+        <v>35</v>
+      </c>
+      <c r="B47">
+        <f>0.63268*10000</f>
+        <v>6326.8</v>
+      </c>
+      <c r="C47">
+        <f t="shared" si="0"/>
+        <v>1.9375505304162481</v>
+      </c>
+      <c r="D47" s="34">
+        <f t="shared" si="1"/>
+        <v>1937.5505304162482</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A48">
+        <v>36</v>
+      </c>
+      <c r="B48" s="33">
+        <f>4/5*B47+1/5*B52</f>
+        <v>6076.2400000000007</v>
+      </c>
+      <c r="C48">
+        <f t="shared" si="0"/>
+        <v>1.8898200076634835</v>
+      </c>
+      <c r="D48" s="34">
+        <f t="shared" si="1"/>
+        <v>1889.8200076634835</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A49">
+        <v>37</v>
+      </c>
+      <c r="B49" s="33">
+        <f>3/5*B47+2/5*B52</f>
+        <v>5825.68</v>
+      </c>
+      <c r="C49">
+        <f t="shared" si="0"/>
+        <v>1.8405780983818707</v>
+      </c>
+      <c r="D49" s="34">
+        <f t="shared" si="1"/>
+        <v>1840.5780983818706</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A50">
+        <v>38</v>
+      </c>
+      <c r="B50" s="33">
+        <f>2/5*B47+3/5*B52</f>
+        <v>5575.1200000000008</v>
+      </c>
+      <c r="C50">
+        <f t="shared" si="0"/>
+        <v>1.7897518606598217</v>
+      </c>
+      <c r="D50" s="34">
+        <f t="shared" si="1"/>
+        <v>1789.7518606598217</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A51">
+        <v>39</v>
+      </c>
+      <c r="B51" s="33">
+        <f>1/5*B47+4/5*B52</f>
+        <v>5324.56</v>
+      </c>
+      <c r="C51">
+        <f t="shared" si="0"/>
+        <v>1.7372635821191604</v>
+      </c>
+      <c r="D51" s="34">
+        <f t="shared" si="1"/>
+        <v>1737.2635821191604</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A52">
+        <v>40</v>
+      </c>
+      <c r="B52">
+        <f>0.5074*10000</f>
+        <v>5074</v>
+      </c>
+      <c r="C52">
+        <f t="shared" si="0"/>
+        <v>1.6830303834416878</v>
+      </c>
+      <c r="D52" s="34">
+        <f t="shared" si="1"/>
+        <v>1683.0303834416877</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A53">
+        <v>41</v>
+      </c>
+      <c r="B53" s="33">
+        <f>4/5*B52+1/5*B57</f>
+        <v>4879.72</v>
+      </c>
+      <c r="C53">
+        <f t="shared" si="0"/>
+        <v>1.6397217151935652</v>
+      </c>
+      <c r="D53" s="34">
+        <f t="shared" si="1"/>
+        <v>1639.7217151935652</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A54">
+        <v>42</v>
+      </c>
+      <c r="B54" s="33">
+        <f>3/5*B52+2/5*B57</f>
+        <v>4685.4400000000005</v>
+      </c>
+      <c r="C54">
+        <f t="shared" si="0"/>
+        <v>1.595267148958424</v>
+      </c>
+      <c r="D54" s="34">
+        <f t="shared" si="1"/>
+        <v>1595.2671489584241</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A55">
+        <v>43</v>
+      </c>
+      <c r="B55" s="33">
+        <f>2/5*B52+3/5*B57</f>
+        <v>4491.16</v>
+      </c>
+      <c r="C55">
+        <f t="shared" si="0"/>
+        <v>1.549620596280767</v>
+      </c>
+      <c r="D55" s="34">
+        <f t="shared" si="1"/>
+        <v>1549.6205962807669</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A56">
+        <v>44</v>
+      </c>
+      <c r="B56" s="33">
+        <f>1/5*B52+4/5*B57</f>
+        <v>4296.88</v>
+      </c>
+      <c r="C56">
+        <f t="shared" si="0"/>
+        <v>1.502733463524909</v>
+      </c>
+      <c r="D56" s="34">
+        <f t="shared" si="1"/>
+        <v>1502.733463524909</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A57">
+        <v>45</v>
+      </c>
+      <c r="B57">
+        <f>0.41026*10000</f>
+        <v>4102.6000000000004</v>
+      </c>
+      <c r="C57">
+        <f t="shared" si="0"/>
+        <v>1.4545544793158709</v>
+      </c>
+      <c r="D57" s="34">
+        <f t="shared" si="1"/>
+        <v>1454.5544793158708</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A58">
+        <v>46</v>
+      </c>
+      <c r="B58" s="33">
+        <f>4/5*B57+1/5*B62</f>
+        <v>3949.34</v>
+      </c>
+      <c r="C58">
+        <f t="shared" si="0"/>
+        <v>1.4156010248513551</v>
+      </c>
+      <c r="D58" s="34">
+        <f t="shared" si="1"/>
+        <v>1415.6010248513551</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A59">
+        <v>47</v>
+      </c>
+      <c r="B59" s="33">
+        <f>3/5*B57+2/5*B62</f>
+        <v>3796.08</v>
+      </c>
+      <c r="C59">
+        <f t="shared" si="0"/>
+        <v>1.3757821062214772</v>
+      </c>
+      <c r="D59" s="34">
+        <f t="shared" si="1"/>
+        <v>1375.7821062214773</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A60">
+        <v>48</v>
+      </c>
+      <c r="B60" s="33">
+        <f>2/5*B57+3/5*B62</f>
+        <v>3642.8199999999997</v>
+      </c>
+      <c r="C60">
+        <f t="shared" si="0"/>
+        <v>1.3350685562075877</v>
+      </c>
+      <c r="D60" s="34">
+        <f t="shared" si="1"/>
+        <v>1335.0685562075878</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A61">
+        <v>49</v>
+      </c>
+      <c r="B61" s="33">
+        <f>1/5*B57+4/5*B62</f>
+        <v>3489.56</v>
+      </c>
+      <c r="C61">
+        <f t="shared" si="0"/>
+        <v>1.2934298820717651</v>
+      </c>
+      <c r="D61" s="34">
+        <f t="shared" si="1"/>
+        <v>1293.4298820717652</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A62">
+        <v>50</v>
+      </c>
+      <c r="B62">
+        <f>0.33363*10000</f>
+        <v>3336.2999999999997</v>
+      </c>
+      <c r="C62">
+        <f t="shared" si="0"/>
+        <v>1.2508341893928601</v>
+      </c>
+      <c r="D62" s="34">
+        <f t="shared" si="1"/>
+        <v>1250.83418939286</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A63">
+        <v>51</v>
+      </c>
+      <c r="B63" s="33">
+        <f>4/5*B62+1/5*B67</f>
+        <v>3213.9</v>
+      </c>
+      <c r="C63">
+        <f t="shared" si="0"/>
+        <v>1.2161057674115894</v>
+      </c>
+      <c r="D63" s="34">
+        <f t="shared" si="1"/>
+        <v>1216.1057674115893</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A64">
+        <v>52</v>
+      </c>
+      <c r="B64" s="33">
+        <f>3/5*B62+2/5*B67</f>
+        <v>3091.5</v>
+      </c>
+      <c r="C64">
+        <f t="shared" si="0"/>
+        <v>1.1807279532521102</v>
+      </c>
+      <c r="D64" s="34">
+        <f t="shared" si="1"/>
+        <v>1180.7279532521102</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A65">
+        <v>53</v>
+      </c>
+      <c r="B65" s="33">
+        <f>2/5*B62+3/5*B67</f>
+        <v>2969.1000000000004</v>
+      </c>
+      <c r="C65">
+        <f t="shared" si="0"/>
+        <v>1.1446823603796716</v>
+      </c>
+      <c r="D65" s="34">
+        <f t="shared" si="1"/>
+        <v>1144.6823603796715</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A66">
+        <v>54</v>
+      </c>
+      <c r="B66" s="33">
+        <f>1/5*B62+4/5*B67</f>
+        <v>2846.7</v>
+      </c>
+      <c r="C66">
+        <f t="shared" si="0"/>
+        <v>1.1079499015311325</v>
+      </c>
+      <c r="D66" s="34">
+        <f t="shared" si="1"/>
+        <v>1107.9499015311326</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A67">
+        <v>55</v>
+      </c>
+      <c r="B67">
+        <f>0.27243*10000</f>
+        <v>2724.3</v>
+      </c>
+      <c r="C67">
+        <f t="shared" ref="C67:C82" si="2">B67/(B67+10000)*5</f>
+        <v>1.0705107550120636</v>
+      </c>
+      <c r="D67" s="34">
+        <f t="shared" ref="D67:D82" si="3">C67*1000</f>
+        <v>1070.5107550120636</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A68">
+        <v>56</v>
+      </c>
+      <c r="B68" s="33">
+        <f>4/5*B67+1/5*B72</f>
+        <v>2626.84</v>
+      </c>
+      <c r="C68">
+        <f t="shared" si="2"/>
+        <v>1.0401810745998208</v>
+      </c>
+      <c r="D68" s="34">
+        <f t="shared" si="3"/>
+        <v>1040.1810745998207</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A69">
+        <v>57</v>
+      </c>
+      <c r="B69" s="33">
+        <f>3/5*B67+2/5*B72</f>
+        <v>2529.38</v>
+      </c>
+      <c r="C69">
+        <f t="shared" si="2"/>
+        <v>1.0093795542955837</v>
+      </c>
+      <c r="D69" s="34">
+        <f t="shared" si="3"/>
+        <v>1009.3795542955837</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A70">
+        <v>58</v>
+      </c>
+      <c r="B70" s="33">
+        <f>2/5*B67+3/5*B72</f>
+        <v>2431.92</v>
+      </c>
+      <c r="C70">
+        <f t="shared" si="2"/>
+        <v>0.97809509713704723</v>
+      </c>
+      <c r="D70" s="34">
+        <f t="shared" si="3"/>
+        <v>978.09509713704722</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A71">
+        <v>59</v>
+      </c>
+      <c r="B71" s="33">
+        <f>1/5*B67+4/5*B72</f>
+        <v>2334.46</v>
+      </c>
+      <c r="C71">
+        <f t="shared" si="2"/>
+        <v>0.94631625543396314</v>
+      </c>
+      <c r="D71" s="34">
+        <f t="shared" si="3"/>
+        <v>946.31625543396319</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A72">
+        <v>60</v>
+      </c>
+      <c r="B72">
+        <f>0.2237*10000</f>
+        <v>2237</v>
+      </c>
+      <c r="C72">
+        <f t="shared" si="2"/>
+        <v>0.91403121680150368</v>
+      </c>
+      <c r="D72" s="34">
+        <f t="shared" si="3"/>
+        <v>914.03121680150366</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A73">
+        <v>61</v>
+      </c>
+      <c r="B73" s="33">
+        <f>4/5*B72+1/5*B77</f>
+        <v>2158.7800000000002</v>
+      </c>
+      <c r="C73">
+        <f t="shared" si="2"/>
+        <v>0.88774531655314115</v>
+      </c>
+      <c r="D73" s="34">
+        <f t="shared" si="3"/>
+        <v>887.74531655314115</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A74">
+        <v>62</v>
+      </c>
+      <c r="B74" s="33">
+        <f>3/5*B72+2/5*B77</f>
+        <v>2080.5600000000004</v>
+      </c>
+      <c r="C74">
+        <f t="shared" si="2"/>
+        <v>0.86111902097253779</v>
+      </c>
+      <c r="D74" s="34">
+        <f t="shared" si="3"/>
+        <v>861.11902097253778</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A75">
+        <v>63</v>
+      </c>
+      <c r="B75" s="33">
+        <f>2/5*B72+3/5*B77</f>
+        <v>2002.3400000000001</v>
+      </c>
+      <c r="C75">
+        <f t="shared" si="2"/>
+        <v>0.83414567492672276</v>
+      </c>
+      <c r="D75" s="34">
+        <f t="shared" si="3"/>
+        <v>834.14567492672279</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A76">
+        <v>64</v>
+      </c>
+      <c r="B76" s="33">
+        <f>1/5*B72+4/5*B77</f>
+        <v>1924.1200000000003</v>
+      </c>
+      <c r="C76">
+        <f t="shared" si="2"/>
+        <v>0.80681844865700791</v>
+      </c>
+      <c r="D76" s="34">
+        <f t="shared" si="3"/>
+        <v>806.81844865700793</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A77">
+        <v>65</v>
+      </c>
+      <c r="B77">
+        <f>0.18459*10000</f>
+        <v>1845.9</v>
+      </c>
+      <c r="C77">
+        <f t="shared" si="2"/>
+        <v>0.77913033201360804</v>
+      </c>
+      <c r="D77" s="34">
+        <f t="shared" si="3"/>
+        <v>779.13033201360804</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A78">
+        <v>66</v>
+      </c>
+      <c r="B78" s="33">
+        <f>4/5*B77+1/5*B82</f>
+        <v>1782.8200000000002</v>
+      </c>
+      <c r="C78">
+        <f t="shared" si="2"/>
+        <v>0.75653366511582121</v>
+      </c>
+      <c r="D78" s="34">
+        <f t="shared" si="3"/>
+        <v>756.53366511582124</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A79">
+        <v>67</v>
+      </c>
+      <c r="B79" s="33">
+        <f>3/5*B77+2/5*B82</f>
+        <v>1719.74</v>
+      </c>
+      <c r="C79">
+        <f t="shared" si="2"/>
+        <v>0.73369375088525857</v>
+      </c>
+      <c r="D79" s="34">
+        <f t="shared" si="3"/>
+        <v>733.69375088525862</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A80">
+        <v>68</v>
+      </c>
+      <c r="B80" s="33">
+        <f>2/5*B77+3/5*B82</f>
+        <v>1656.66</v>
+      </c>
+      <c r="C80">
+        <f t="shared" si="2"/>
+        <v>0.71060664032407228</v>
+      </c>
+      <c r="D80" s="34">
+        <f t="shared" si="3"/>
+        <v>710.60664032407226</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A81">
+        <v>69</v>
+      </c>
+      <c r="B81" s="33">
+        <f>1/5*B77+4/5*B82</f>
+        <v>1593.5800000000002</v>
+      </c>
+      <c r="C81">
+        <f t="shared" si="2"/>
+        <v>0.68726829848933635</v>
+      </c>
+      <c r="D81" s="34">
+        <f t="shared" si="3"/>
+        <v>687.2682984893363</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A82">
+        <v>70</v>
+      </c>
+      <c r="B82">
+        <f>0.15305*10000</f>
+        <v>1530.5</v>
+      </c>
+      <c r="C82">
+        <f t="shared" si="2"/>
+        <v>0.66367460214214469</v>
+      </c>
+      <c r="D82" s="34">
+        <f t="shared" si="3"/>
+        <v>663.67460214214464</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{b75eb9d1-7479-4f8a-9240-cc5b19dbbc64}" enabled="1" method="Standard" siteId="{d1b36e95-0d50-42e9-958f-b63fa906beaa}" removed="0"/>

</xml_diff>

<commit_message>
Extended temperature lookup table in Excel and code
</commit_message>
<xml_diff>
--- a/Excel/sensors.xlsx
+++ b/Excel/sensors.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uoa-my.sharepoint.com/personal/ctra157_uoa_auckland_ac_nz/Documents/Documents/GitHub/311/Excel/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ctra157\Documents\GitHub\311\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="208" documentId="13_ncr:1_{FEF83167-29AA-4D2C-9F19-8FB03B27FB56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{89A6A94C-C3E5-4D4D-B720-7A07230B4FEB}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83C5B04E-D882-4E3B-A5CB-20935787FB49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="649" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -860,9 +860,8 @@
     <xf numFmtId="167" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -881,8 +880,9 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1730,24 +1730,24 @@
       <c r="K3" s="1"/>
     </row>
     <row r="4" spans="2:17" ht="73.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="27"/>
-      <c r="C4" s="27"/>
-      <c r="D4" s="27"/>
-      <c r="E4" s="27"/>
+      <c r="B4" s="28"/>
+      <c r="C4" s="28"/>
+      <c r="D4" s="28"/>
+      <c r="E4" s="28"/>
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
-      <c r="H4" s="29" t="s">
+      <c r="H4" s="30" t="s">
         <v>4</v>
       </c>
-      <c r="I4" s="30"/>
-      <c r="J4" s="30"/>
-      <c r="K4" s="30"/>
-      <c r="N4" s="28" t="s">
+      <c r="I4" s="31"/>
+      <c r="J4" s="31"/>
+      <c r="K4" s="31"/>
+      <c r="N4" s="29" t="s">
         <v>5</v>
       </c>
-      <c r="O4" s="28"/>
-      <c r="P4" s="28"/>
-      <c r="Q4" s="28"/>
+      <c r="O4" s="29"/>
+      <c r="P4" s="29"/>
+      <c r="Q4" s="29"/>
     </row>
     <row r="5" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="10" t="s">
@@ -2370,12 +2370,12 @@
       <c r="Q10" s="10"/>
     </row>
     <row r="11" spans="2:17" ht="99.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="N11" s="31" t="s">
+      <c r="N11" s="32" t="s">
         <v>121</v>
       </c>
-      <c r="O11" s="31"/>
-      <c r="P11" s="31"/>
-      <c r="Q11" s="31"/>
+      <c r="O11" s="32"/>
+      <c r="P11" s="32"/>
+      <c r="Q11" s="32"/>
     </row>
     <row r="12" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="N12" s="10" t="s">
@@ -2719,15 +2719,15 @@
       </c>
     </row>
     <row r="15" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="32" t="s">
+      <c r="B15" s="33" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="16" spans="2:17" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="32"/>
+      <c r="B16" s="33"/>
     </row>
     <row r="17" spans="2:6" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="32"/>
+      <c r="B17" s="33"/>
       <c r="F17"/>
     </row>
   </sheetData>
@@ -2770,25 +2770,25 @@
       <c r="S1" s="15"/>
     </row>
     <row r="2" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="26" t="s">
+      <c r="B2" s="34" t="s">
         <v>68</v>
       </c>
-      <c r="C2" s="26"/>
-      <c r="D2" s="26" t="s">
+      <c r="C2" s="34"/>
+      <c r="D2" s="34" t="s">
         <v>69</v>
       </c>
-      <c r="E2" s="26"/>
-      <c r="F2" s="26" t="s">
+      <c r="E2" s="34"/>
+      <c r="F2" s="34" t="s">
         <v>70</v>
       </c>
-      <c r="G2" s="26"/>
+      <c r="G2" s="34"/>
       <c r="H2" s="10"/>
-      <c r="I2" s="26" t="s">
+      <c r="I2" s="34" t="s">
         <v>80</v>
       </c>
-      <c r="J2" s="26"/>
-      <c r="K2" s="26"/>
-      <c r="L2" s="26"/>
+      <c r="J2" s="34"/>
+      <c r="K2" s="34"/>
+      <c r="L2" s="34"/>
     </row>
     <row r="3" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="10" t="s">
@@ -2809,14 +2809,14 @@
       <c r="G3" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="I3" s="26" t="s">
+      <c r="I3" s="34" t="s">
         <v>67</v>
       </c>
-      <c r="J3" s="26"/>
-      <c r="K3" s="26" t="s">
+      <c r="J3" s="34"/>
+      <c r="K3" s="34" t="s">
         <v>71</v>
       </c>
-      <c r="L3" s="26"/>
+      <c r="L3" s="34"/>
     </row>
     <row r="4" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
@@ -2935,24 +2935,24 @@
       <c r="S7" s="1"/>
     </row>
     <row r="8" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="26" t="s">
+      <c r="B8" s="34" t="s">
         <v>68</v>
       </c>
-      <c r="C8" s="26"/>
-      <c r="D8" s="26"/>
-      <c r="E8" s="26"/>
-      <c r="F8" s="26" t="s">
+      <c r="C8" s="34"/>
+      <c r="D8" s="34"/>
+      <c r="E8" s="34"/>
+      <c r="F8" s="34" t="s">
         <v>69</v>
       </c>
-      <c r="G8" s="26"/>
-      <c r="H8" s="26"/>
-      <c r="I8" s="26"/>
-      <c r="J8" s="26" t="s">
+      <c r="G8" s="34"/>
+      <c r="H8" s="34"/>
+      <c r="I8" s="34"/>
+      <c r="J8" s="34" t="s">
         <v>70</v>
       </c>
-      <c r="K8" s="26"/>
-      <c r="L8" s="26"/>
-      <c r="M8" s="26"/>
+      <c r="K8" s="34"/>
+      <c r="L8" s="34"/>
+      <c r="M8" s="34"/>
       <c r="N8" s="1"/>
       <c r="O8" s="1"/>
       <c r="P8" s="1"/>
@@ -2961,30 +2961,30 @@
       <c r="S8" s="1"/>
     </row>
     <row r="9" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="26" t="s">
+      <c r="B9" s="34" t="s">
         <v>67</v>
       </c>
-      <c r="C9" s="26"/>
-      <c r="D9" s="26" t="s">
+      <c r="C9" s="34"/>
+      <c r="D9" s="34" t="s">
         <v>71</v>
       </c>
-      <c r="E9" s="26"/>
-      <c r="F9" s="26" t="s">
+      <c r="E9" s="34"/>
+      <c r="F9" s="34" t="s">
         <v>67</v>
       </c>
-      <c r="G9" s="26"/>
-      <c r="H9" s="26" t="s">
+      <c r="G9" s="34"/>
+      <c r="H9" s="34" t="s">
         <v>71</v>
       </c>
-      <c r="I9" s="26"/>
-      <c r="J9" s="26" t="s">
+      <c r="I9" s="34"/>
+      <c r="J9" s="34" t="s">
         <v>67</v>
       </c>
-      <c r="K9" s="26"/>
-      <c r="L9" s="26" t="s">
+      <c r="K9" s="34"/>
+      <c r="L9" s="34" t="s">
         <v>71</v>
       </c>
-      <c r="M9" s="26"/>
+      <c r="M9" s="34"/>
     </row>
     <row r="10" spans="1:19" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="1" t="s">
@@ -3096,18 +3096,18 @@
       </c>
     </row>
     <row r="18" spans="2:8" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="26" t="s">
+      <c r="B18" s="34" t="s">
         <v>68</v>
       </c>
-      <c r="C18" s="26"/>
-      <c r="D18" s="26" t="s">
+      <c r="C18" s="34"/>
+      <c r="D18" s="34" t="s">
         <v>69</v>
       </c>
-      <c r="E18" s="26"/>
-      <c r="F18" s="26" t="s">
+      <c r="E18" s="34"/>
+      <c r="F18" s="34" t="s">
         <v>70</v>
       </c>
-      <c r="G18" s="26"/>
+      <c r="G18" s="34"/>
     </row>
     <row r="19" spans="2:8" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="1" t="s">
@@ -3176,6 +3176,12 @@
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="D18:E18"/>
+    <mergeCell ref="F18:G18"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="F2:G2"/>
     <mergeCell ref="I2:L2"/>
     <mergeCell ref="I3:J3"/>
     <mergeCell ref="K3:L3"/>
@@ -3188,12 +3194,6 @@
     <mergeCell ref="H9:I9"/>
     <mergeCell ref="J9:K9"/>
     <mergeCell ref="L9:M9"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="D18:E18"/>
-    <mergeCell ref="F18:G18"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="F2:G2"/>
   </mergeCells>
   <phoneticPr fontId="11" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3714,7 +3714,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A1B340A-C562-401C-9C12-DAC3640D6A6E}">
-  <dimension ref="A1:F82"/>
+  <dimension ref="A1:F102"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.28515625" customWidth="1"/>
@@ -3738,1382 +3738,1718 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2">
+        <v>-20</v>
+      </c>
+      <c r="B2">
+        <v>114660</v>
+      </c>
+      <c r="C2">
+        <f>B2/(B2+10000)*5</f>
+        <v>4.5989090325685869</v>
+      </c>
+      <c r="D2" s="27">
+        <f>C2*1000</f>
+        <v>4598.9090325685866</v>
+      </c>
+      <c r="F2" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>-19</v>
+      </c>
+      <c r="B3" s="26">
+        <f>4/5*B2+1/5*B7</f>
+        <v>108630</v>
+      </c>
+      <c r="C3">
+        <f t="shared" ref="C3:C6" si="0">B3/(B3+10000)*5</f>
+        <v>4.5785214532580296</v>
+      </c>
+      <c r="D3" s="27">
+        <f t="shared" ref="D3:D6" si="1">C3*1000</f>
+        <v>4578.5214532580294</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>-18</v>
+      </c>
+      <c r="B4" s="26">
+        <f>3/5*B2+2/5*B7</f>
+        <v>102600</v>
+      </c>
+      <c r="C4">
+        <f t="shared" si="0"/>
+        <v>4.5559502664298401</v>
+      </c>
+      <c r="D4" s="27">
+        <f t="shared" si="1"/>
+        <v>4555.9502664298398</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>-17</v>
+      </c>
+      <c r="B5" s="26">
+        <f>2/5*B2+3/5*B7</f>
+        <v>96570</v>
+      </c>
+      <c r="C5">
+        <f t="shared" si="0"/>
+        <v>4.5308248099840478</v>
+      </c>
+      <c r="D5" s="27">
+        <f t="shared" si="1"/>
+        <v>4530.8248099840475</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>-16</v>
+      </c>
+      <c r="B6" s="26">
+        <f>1/5*B2+4/5*B7</f>
+        <v>90540</v>
+      </c>
+      <c r="C6">
+        <f t="shared" si="0"/>
+        <v>4.5026854983091305</v>
+      </c>
+      <c r="D6" s="27">
+        <f t="shared" si="1"/>
+        <v>4502.6854983091307</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>-15</v>
+      </c>
+      <c r="B7">
+        <v>84510</v>
+      </c>
+      <c r="C7">
+        <f>B7/(B7+10000)*5</f>
+        <v>4.4709554544492649</v>
+      </c>
+      <c r="D7" s="27">
+        <f>C7*1000</f>
+        <v>4470.9554544492648</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>-14</v>
+      </c>
+      <c r="B8" s="26">
+        <f>4/5*B7+1/5*B12</f>
+        <v>80193.399999999994</v>
+      </c>
+      <c r="C8">
+        <f t="shared" ref="C8:C11" si="2">B8/(B8+10000)*5</f>
+        <v>4.4456357117039609</v>
+      </c>
+      <c r="D8" s="27">
+        <f t="shared" ref="D8:D11" si="3">C8*1000</f>
+        <v>4445.6357117039606</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>-13</v>
+      </c>
+      <c r="B9" s="26">
+        <f>3/5*B7+2/5*B12</f>
+        <v>75876.800000000003</v>
+      </c>
+      <c r="C9">
+        <f t="shared" si="2"/>
+        <v>4.4177705736590092</v>
+      </c>
+      <c r="D9" s="27">
+        <f t="shared" si="3"/>
+        <v>4417.7705736590087</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>-12</v>
+      </c>
+      <c r="B10" s="26">
+        <f>2/5*B7+3/5*B12</f>
+        <v>71560.2</v>
+      </c>
+      <c r="C10">
+        <f t="shared" si="2"/>
+        <v>4.3869558927025682</v>
+      </c>
+      <c r="D10" s="27">
+        <f t="shared" si="3"/>
+        <v>4386.9558927025682</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>-11</v>
+      </c>
+      <c r="B11" s="26">
+        <f>1/5*B7+4/5*B12</f>
+        <v>67243.600000000006</v>
+      </c>
+      <c r="C11">
+        <f t="shared" si="2"/>
+        <v>4.3526971813846069</v>
+      </c>
+      <c r="D11" s="27">
+        <f t="shared" si="3"/>
+        <v>4352.6971813846067</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12">
         <v>-10</v>
       </c>
-      <c r="B2">
+      <c r="B12">
         <f>6.2927*10000</f>
         <v>62927</v>
       </c>
-      <c r="C2">
-        <f>B2/(B2+10000)*5</f>
+      <c r="C12">
+        <f>B12/(B12+10000)*5</f>
         <v>4.3143828760267118</v>
       </c>
-      <c r="D2" s="34">
-        <f>C2*1000</f>
+      <c r="D12" s="27">
+        <f>C12*1000</f>
         <v>4314.3828760267115</v>
       </c>
-      <c r="F2" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3">
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13">
         <v>-9</v>
       </c>
-      <c r="B3" s="33">
-        <f>4/5*B2+1/5*B7</f>
+      <c r="B13" s="26">
+        <f>4/5*B12+1/5*B17</f>
         <v>59757.000000000007</v>
       </c>
-      <c r="C3">
-        <f t="shared" ref="C3:C66" si="0">B3/(B3+10000)*5</f>
+      <c r="C13">
+        <f t="shared" ref="C13:C76" si="4">B13/(B13+10000)*5</f>
         <v>4.2832260561664066</v>
       </c>
-      <c r="D3" s="34">
-        <f t="shared" ref="D3:D66" si="1">C3*1000</f>
+      <c r="D13" s="27">
+        <f t="shared" ref="D13:D76" si="5">C13*1000</f>
         <v>4283.226056166407</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14">
         <v>-8</v>
       </c>
-      <c r="B4" s="33">
-        <f>3/5*B2+2/5*B7</f>
+      <c r="B14" s="26">
+        <f>3/5*B12+2/5*B17</f>
         <v>56587</v>
       </c>
-      <c r="C4">
-        <f t="shared" si="0"/>
+      <c r="C14">
+        <f t="shared" si="4"/>
         <v>4.2491026776998515</v>
       </c>
-      <c r="D4" s="34">
-        <f t="shared" si="1"/>
+      <c r="D14" s="27">
+        <f t="shared" si="5"/>
         <v>4249.1026776998515</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15">
         <v>-7</v>
       </c>
-      <c r="B5" s="33">
-        <f>2/5*B2+3/5*B7</f>
+      <c r="B15" s="26">
+        <f>2/5*B12+3/5*B17</f>
         <v>53417</v>
       </c>
-      <c r="C5">
-        <f t="shared" si="0"/>
+      <c r="C15">
+        <f t="shared" si="4"/>
         <v>4.2115678761215447</v>
       </c>
-      <c r="D5" s="34">
-        <f t="shared" si="1"/>
+      <c r="D15" s="27">
+        <f t="shared" si="5"/>
         <v>4211.5678761215449</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16">
         <v>-6</v>
       </c>
-      <c r="B6" s="33">
-        <f>1/5*B2+4/5*B7</f>
+      <c r="B16" s="26">
+        <f>1/5*B12+4/5*B17</f>
         <v>50247</v>
       </c>
-      <c r="C6">
-        <f t="shared" si="0"/>
+      <c r="C16">
+        <f t="shared" si="4"/>
         <v>4.1700831576676016</v>
       </c>
-      <c r="D6" s="34">
-        <f t="shared" si="1"/>
+      <c r="D16" s="27">
+        <f t="shared" si="5"/>
         <v>4170.0831576676019</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17">
         <v>-5</v>
       </c>
-      <c r="B7">
+      <c r="B17">
         <f>4.7077*10000</f>
         <v>47077</v>
       </c>
-      <c r="C7">
-        <f t="shared" si="0"/>
+      <c r="C17">
+        <f t="shared" si="4"/>
         <v>4.1239903989347724</v>
       </c>
-      <c r="D7" s="34">
-        <f t="shared" si="1"/>
+      <c r="D17" s="27">
+        <f t="shared" si="5"/>
         <v>4123.9903989347722</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18">
         <v>-4</v>
       </c>
-      <c r="B8" s="33">
-        <f>4/5*B7+1/5*B12</f>
+      <c r="B18" s="26">
+        <f>4/5*B17+1/5*B22</f>
         <v>44774.2</v>
       </c>
-      <c r="C8">
-        <f t="shared" si="0"/>
+      <c r="C18">
+        <f t="shared" si="4"/>
         <v>4.0871614738325706</v>
       </c>
-      <c r="D8" s="34">
-        <f t="shared" si="1"/>
+      <c r="D18" s="27">
+        <f t="shared" si="5"/>
         <v>4087.1614738325707</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19">
         <v>-3</v>
       </c>
-      <c r="B9" s="33">
-        <f>3/5*B7+2/5*B12</f>
+      <c r="B19" s="26">
+        <f>3/5*B17+2/5*B22</f>
         <v>42471.4</v>
       </c>
-      <c r="C9">
-        <f t="shared" si="0"/>
+      <c r="C19">
+        <f t="shared" si="4"/>
         <v>4.0470999439694761</v>
       </c>
-      <c r="D9" s="34">
-        <f t="shared" si="1"/>
+      <c r="D19" s="27">
+        <f t="shared" si="5"/>
         <v>4047.099943969476</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20">
         <v>-2</v>
       </c>
-      <c r="B10" s="33">
-        <f>2/5*B7+3/5*B12</f>
+      <c r="B20" s="26">
+        <f>2/5*B17+3/5*B22</f>
         <v>40168.6</v>
       </c>
-      <c r="C10">
-        <f t="shared" si="0"/>
+      <c r="C20">
+        <f t="shared" si="4"/>
         <v>4.0033606678280833</v>
       </c>
-      <c r="D10" s="34">
-        <f t="shared" si="1"/>
+      <c r="D20" s="27">
+        <f t="shared" si="5"/>
         <v>4003.3606678280835</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21">
         <v>-1</v>
       </c>
-      <c r="B11" s="33">
-        <f>1/5*B7+4/5*B12</f>
+      <c r="B21" s="26">
+        <f>1/5*B17+4/5*B22</f>
         <v>37865.800000000003</v>
       </c>
-      <c r="C11">
-        <f t="shared" si="0"/>
+      <c r="C21">
+        <f t="shared" si="4"/>
         <v>3.9554128417366892</v>
       </c>
-      <c r="D11" s="34">
-        <f t="shared" si="1"/>
+      <c r="D21" s="27">
+        <f t="shared" si="5"/>
         <v>3955.4128417366892</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22">
         <v>0</v>
       </c>
-      <c r="B12">
+      <c r="B22">
         <f>3.5563*10000</f>
         <v>35563</v>
       </c>
-      <c r="C12">
-        <f t="shared" si="0"/>
+      <c r="C22">
+        <f t="shared" si="4"/>
         <v>3.9026183526106712</v>
       </c>
-      <c r="D12" s="34">
-        <f t="shared" si="1"/>
+      <c r="D22" s="27">
+        <f t="shared" si="5"/>
         <v>3902.6183526106711</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23">
         <v>1</v>
       </c>
-      <c r="B13" s="33">
-        <f>4/5*B12+1/5*B17</f>
+      <c r="B23" s="26">
+        <f>4/5*B22+1/5*B27</f>
         <v>33874.200000000004</v>
       </c>
-      <c r="C13">
-        <f t="shared" si="0"/>
+      <c r="C23">
+        <f t="shared" si="4"/>
         <v>3.8603780809678585</v>
       </c>
-      <c r="D13" s="34">
-        <f t="shared" si="1"/>
+      <c r="D23" s="27">
+        <f t="shared" si="5"/>
         <v>3860.3780809678583</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24">
         <v>2</v>
       </c>
-      <c r="B14" s="33">
-        <f>3/5*B12+2/5*B17</f>
+      <c r="B24" s="26">
+        <f>3/5*B22+2/5*B27</f>
         <v>32185.4</v>
       </c>
-      <c r="C14">
-        <f t="shared" si="0"/>
+      <c r="C24">
+        <f t="shared" si="4"/>
         <v>3.8147558159932111</v>
       </c>
-      <c r="D14" s="34">
-        <f t="shared" si="1"/>
+      <c r="D24" s="27">
+        <f t="shared" si="5"/>
         <v>3814.7558159932109</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25">
         <v>3</v>
       </c>
-      <c r="B15" s="33">
-        <f>2/5*B12+3/5*B17</f>
+      <c r="B25" s="26">
+        <f>2/5*B22+3/5*B27</f>
         <v>30496.6</v>
       </c>
-      <c r="C15">
-        <f t="shared" si="0"/>
+      <c r="C25">
+        <f t="shared" si="4"/>
         <v>3.7653284473264419</v>
       </c>
-      <c r="D15" s="34">
-        <f t="shared" si="1"/>
+      <c r="D25" s="27">
+        <f t="shared" si="5"/>
         <v>3765.3284473264421</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26">
         <v>4</v>
       </c>
-      <c r="B16" s="33">
-        <f>1/5*B12+4/5*B17</f>
+      <c r="B26" s="26">
+        <f>1/5*B22+4/5*B27</f>
         <v>28807.800000000003</v>
       </c>
-      <c r="C16">
-        <f t="shared" si="0"/>
+      <c r="C26">
+        <f t="shared" si="4"/>
         <v>3.7115992145908812</v>
       </c>
-      <c r="D16" s="34">
-        <f t="shared" si="1"/>
+      <c r="D26" s="27">
+        <f t="shared" si="5"/>
         <v>3711.5992145908813</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27">
         <v>5</v>
       </c>
-      <c r="B17">
+      <c r="B27">
         <f>2.7119*10000</f>
         <v>27119</v>
       </c>
-      <c r="C17">
-        <f t="shared" si="0"/>
+      <c r="C27">
+        <f t="shared" si="4"/>
         <v>3.6529809531506774</v>
       </c>
-      <c r="D17" s="34">
-        <f t="shared" si="1"/>
+      <c r="D27" s="27">
+        <f t="shared" si="5"/>
         <v>3652.9809531506776</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28">
         <v>6</v>
       </c>
-      <c r="B18" s="33">
-        <f>4/5*B17+1/5*B22</f>
+      <c r="B28" s="26">
+        <f>4/5*B27+1/5*B32</f>
         <v>25867.200000000001</v>
       </c>
-      <c r="C18">
-        <f t="shared" si="0"/>
+      <c r="C28">
+        <f t="shared" si="4"/>
         <v>3.6059686844805281</v>
       </c>
-      <c r="D18" s="34">
-        <f t="shared" si="1"/>
+      <c r="D28" s="27">
+        <f t="shared" si="5"/>
         <v>3605.9686844805283</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29">
         <v>7</v>
       </c>
-      <c r="B19" s="33">
-        <f>3/5*B17+2/5*B22</f>
+      <c r="B29" s="26">
+        <f>3/5*B27+2/5*B32</f>
         <v>24615.4</v>
       </c>
-      <c r="C19">
-        <f t="shared" si="0"/>
+      <c r="C29">
+        <f t="shared" si="4"/>
         <v>3.5555561975305787</v>
       </c>
-      <c r="D19" s="34">
-        <f t="shared" si="1"/>
+      <c r="D29" s="27">
+        <f t="shared" si="5"/>
         <v>3555.5561975305786</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30">
         <v>8</v>
       </c>
-      <c r="B20" s="33">
-        <f>2/5*B17+3/5*B22</f>
+      <c r="B30" s="26">
+        <f>2/5*B27+3/5*B32</f>
         <v>23363.599999999999</v>
       </c>
-      <c r="C20">
-        <f t="shared" si="0"/>
+      <c r="C30">
+        <f t="shared" si="4"/>
         <v>3.5013607644259008</v>
       </c>
-      <c r="D20" s="34">
-        <f t="shared" si="1"/>
+      <c r="D30" s="27">
+        <f t="shared" si="5"/>
         <v>3501.3607644259009</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31">
         <v>9</v>
       </c>
-      <c r="B21" s="33">
-        <f>1/5*B17+4/5*B22</f>
+      <c r="B31" s="26">
+        <f>1/5*B27+4/5*B32</f>
         <v>22111.8</v>
       </c>
-      <c r="C21">
-        <f t="shared" si="0"/>
+      <c r="C31">
+        <f t="shared" si="4"/>
         <v>3.4429399784502897</v>
       </c>
-      <c r="D21" s="34">
-        <f t="shared" si="1"/>
+      <c r="D31" s="27">
+        <f t="shared" si="5"/>
         <v>3442.9399784502898</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32">
         <v>10</v>
       </c>
-      <c r="B22">
+      <c r="B32">
         <f>2.086*10000</f>
         <v>20860</v>
       </c>
-      <c r="C22">
-        <f t="shared" si="0"/>
+      <c r="C32">
+        <f t="shared" si="4"/>
         <v>3.3797796500324044</v>
       </c>
-      <c r="D22" s="34">
-        <f t="shared" si="1"/>
+      <c r="D32" s="27">
+        <f t="shared" si="5"/>
         <v>3379.7796500324043</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A33">
         <v>11</v>
       </c>
-      <c r="B23" s="33">
-        <f>4/5*B22+1/5*B27</f>
+      <c r="B33" s="26">
+        <f>4/5*B32+1/5*B37</f>
         <v>19928.8</v>
       </c>
-      <c r="C23">
-        <f t="shared" si="0"/>
+      <c r="C33">
+        <f t="shared" si="4"/>
         <v>3.3293683675924193</v>
       </c>
-      <c r="D23" s="34">
-        <f t="shared" si="1"/>
+      <c r="D33" s="27">
+        <f t="shared" si="5"/>
         <v>3329.3683675924194</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A34">
         <v>12</v>
       </c>
-      <c r="B24" s="33">
-        <f>3/5*B22+2/5*B27</f>
+      <c r="B34" s="26">
+        <f>3/5*B32+2/5*B37</f>
         <v>18997.599999999999</v>
       </c>
-      <c r="C24">
-        <f t="shared" si="0"/>
+      <c r="C34">
+        <f t="shared" si="4"/>
         <v>3.2757193698788867</v>
       </c>
-      <c r="D24" s="34">
-        <f t="shared" si="1"/>
+      <c r="D34" s="27">
+        <f t="shared" si="5"/>
         <v>3275.7193698788865</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A35">
         <v>13</v>
       </c>
-      <c r="B25" s="33">
-        <f>2/5*B22+3/5*B27</f>
+      <c r="B35" s="26">
+        <f>2/5*B32+3/5*B37</f>
         <v>18066.400000000001</v>
       </c>
-      <c r="C25">
-        <f t="shared" si="0"/>
+      <c r="C35">
+        <f t="shared" si="4"/>
         <v>3.2185103896474079</v>
       </c>
-      <c r="D25" s="34">
-        <f t="shared" si="1"/>
+      <c r="D35" s="27">
+        <f t="shared" si="5"/>
         <v>3218.5103896474079</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36">
         <v>14</v>
       </c>
-      <c r="B26" s="33">
-        <f>1/5*B22+4/5*B27</f>
+      <c r="B36" s="26">
+        <f>1/5*B32+4/5*B37</f>
         <v>17135.2</v>
       </c>
-      <c r="C26">
-        <f t="shared" si="0"/>
+      <c r="C36">
+        <f t="shared" si="4"/>
         <v>3.1573749226097467</v>
       </c>
-      <c r="D26" s="34">
-        <f t="shared" si="1"/>
+      <c r="D36" s="27">
+        <f t="shared" si="5"/>
         <v>3157.3749226097466</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A37">
         <v>15</v>
       </c>
-      <c r="B27">
+      <c r="B37">
         <f>1.6204*10000</f>
         <v>16204</v>
       </c>
-      <c r="C27">
-        <f t="shared" si="0"/>
+      <c r="C37">
+        <f t="shared" si="4"/>
         <v>3.0918943672721722</v>
       </c>
-      <c r="D27" s="34">
-        <f t="shared" si="1"/>
+      <c r="D37" s="27">
+        <f t="shared" si="5"/>
         <v>3091.8943672721721</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A38">
         <v>16</v>
       </c>
-      <c r="B28" s="33">
-        <f>4/5*B27+1/5*B32</f>
+      <c r="B38" s="26">
+        <f>4/5*B37+1/5*B42</f>
         <v>15499.800000000001</v>
       </c>
-      <c r="C28">
-        <f t="shared" si="0"/>
+      <c r="C38">
+        <f t="shared" si="4"/>
         <v>3.0392003074533918</v>
       </c>
-      <c r="D28" s="34">
-        <f t="shared" si="1"/>
+      <c r="D38" s="27">
+        <f t="shared" si="5"/>
         <v>3039.2003074533918</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A39">
         <v>17</v>
       </c>
-      <c r="B29" s="33">
-        <f>3/5*B27+2/5*B32</f>
+      <c r="B39" s="26">
+        <f>3/5*B37+2/5*B42</f>
         <v>14795.6</v>
       </c>
-      <c r="C29">
-        <f t="shared" si="0"/>
+      <c r="C39">
+        <f t="shared" si="4"/>
         <v>2.9835132039555408</v>
       </c>
-      <c r="D29" s="34">
-        <f t="shared" si="1"/>
+      <c r="D39" s="27">
+        <f t="shared" si="5"/>
         <v>2983.5132039555406</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A40">
         <v>18</v>
       </c>
-      <c r="B30" s="33">
-        <f>2/5*B27+3/5*B32</f>
+      <c r="B40" s="26">
+        <f>2/5*B37+3/5*B42</f>
         <v>14091.4</v>
       </c>
-      <c r="C30">
-        <f t="shared" si="0"/>
+      <c r="C40">
+        <f t="shared" si="4"/>
         <v>2.9245705936558268</v>
       </c>
-      <c r="D30" s="34">
-        <f t="shared" si="1"/>
+      <c r="D40" s="27">
+        <f t="shared" si="5"/>
         <v>2924.570593655827</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A41">
         <v>19</v>
       </c>
-      <c r="B31" s="33">
-        <f>1/5*B27+4/5*B32</f>
+      <c r="B41" s="26">
+        <f>1/5*B37+4/5*B42</f>
         <v>13387.2</v>
       </c>
-      <c r="C31">
-        <f t="shared" si="0"/>
+      <c r="C41">
+        <f t="shared" si="4"/>
         <v>2.8620784018608472</v>
       </c>
-      <c r="D31" s="34">
-        <f t="shared" si="1"/>
+      <c r="D41" s="27">
+        <f t="shared" si="5"/>
         <v>2862.078401860847</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A42">
         <v>20</v>
       </c>
-      <c r="B32">
+      <c r="B42">
         <f>1.2683*10000</f>
         <v>12683</v>
       </c>
-      <c r="C32">
-        <f t="shared" si="0"/>
+      <c r="C42">
+        <f t="shared" si="4"/>
         <v>2.7957060353568752</v>
       </c>
-      <c r="D32" s="34">
-        <f t="shared" si="1"/>
+      <c r="D42" s="27">
+        <f t="shared" si="5"/>
         <v>2795.7060353568754</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A43">
         <v>21</v>
       </c>
-      <c r="B33" s="33">
-        <f>4/5*B32+1/5*B37</f>
+      <c r="B43" s="26">
+        <f>4/5*B42+1/5*B47</f>
         <v>12146.400000000001</v>
       </c>
-      <c r="C33">
-        <f t="shared" si="0"/>
+      <c r="C43">
+        <f t="shared" si="4"/>
         <v>2.7422967163963445</v>
       </c>
-      <c r="D33" s="34">
-        <f t="shared" si="1"/>
+      <c r="D43" s="27">
+        <f t="shared" si="5"/>
         <v>2742.2967163963444</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A44">
         <v>22</v>
       </c>
-      <c r="B34" s="33">
-        <f>3/5*B32+2/5*B37</f>
+      <c r="B44" s="26">
+        <f>3/5*B42+2/5*B47</f>
         <v>11609.8</v>
       </c>
-      <c r="C34">
-        <f t="shared" si="0"/>
+      <c r="C44">
+        <f t="shared" si="4"/>
         <v>2.6862349489583432</v>
       </c>
-      <c r="D34" s="34">
-        <f t="shared" si="1"/>
+      <c r="D44" s="27">
+        <f t="shared" si="5"/>
         <v>2686.2349489583435</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A45">
         <v>23</v>
       </c>
-      <c r="B35" s="33">
-        <f>2/5*B32+3/5*B37</f>
+      <c r="B45" s="26">
+        <f>2/5*B42+3/5*B47</f>
         <v>11073.2</v>
       </c>
-      <c r="C35">
-        <f t="shared" si="0"/>
+      <c r="C45">
+        <f t="shared" si="4"/>
         <v>2.6273181102063288</v>
       </c>
-      <c r="D35" s="34">
-        <f t="shared" si="1"/>
+      <c r="D45" s="27">
+        <f t="shared" si="5"/>
         <v>2627.3181102063286</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A46">
         <v>24</v>
       </c>
-      <c r="B36" s="33">
-        <f>1/5*B32+4/5*B37</f>
+      <c r="B46" s="26">
+        <f>1/5*B42+4/5*B47</f>
         <v>10536.6</v>
       </c>
-      <c r="C36">
-        <f t="shared" si="0"/>
+      <c r="C46">
+        <f t="shared" si="4"/>
         <v>2.5653224000077914</v>
       </c>
-      <c r="D36" s="34">
-        <f t="shared" si="1"/>
+      <c r="D46" s="27">
+        <f t="shared" si="5"/>
         <v>2565.3224000077917</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A47">
         <v>25</v>
       </c>
-      <c r="B37">
+      <c r="B47">
         <f>10000</f>
         <v>10000</v>
       </c>
-      <c r="C37">
-        <f t="shared" si="0"/>
+      <c r="C47">
+        <f t="shared" si="4"/>
         <v>2.5</v>
       </c>
-      <c r="D37" s="34">
-        <f t="shared" si="1"/>
+      <c r="D47" s="27">
+        <f t="shared" si="5"/>
         <v>2500</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A48">
         <v>26</v>
       </c>
-      <c r="B38" s="33">
-        <f>4/5*B37+1/5*B42</f>
+      <c r="B48" s="26">
+        <f>4/5*B47+1/5*B52</f>
         <v>9588.4</v>
       </c>
-      <c r="C38">
-        <f t="shared" si="0"/>
+      <c r="C48">
+        <f t="shared" si="4"/>
         <v>2.4474689101713256</v>
       </c>
-      <c r="D38" s="34">
-        <f t="shared" si="1"/>
+      <c r="D48" s="27">
+        <f t="shared" si="5"/>
         <v>2447.4689101713257</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A49">
         <v>27</v>
       </c>
-      <c r="B39" s="33">
-        <f>3/5*B37+2/5*B42</f>
+      <c r="B49" s="26">
+        <f>3/5*B47+2/5*B52</f>
         <v>9176.7999999999993</v>
       </c>
-      <c r="C39">
-        <f t="shared" si="0"/>
+      <c r="C49">
+        <f t="shared" si="4"/>
         <v>2.3926828250803052</v>
       </c>
-      <c r="D39" s="34">
-        <f t="shared" si="1"/>
+      <c r="D49" s="27">
+        <f t="shared" si="5"/>
         <v>2392.6828250803051</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A50">
         <v>28</v>
       </c>
-      <c r="B40" s="33">
-        <f>2/5*B37+3/5*B42</f>
+      <c r="B50" s="26">
+        <f>2/5*B47+3/5*B52</f>
         <v>8765.2000000000007</v>
       </c>
-      <c r="C40">
-        <f t="shared" si="0"/>
+      <c r="C50">
+        <f t="shared" si="4"/>
         <v>2.3354933600494534</v>
       </c>
-      <c r="D40" s="34">
-        <f t="shared" si="1"/>
+      <c r="D50" s="27">
+        <f t="shared" si="5"/>
         <v>2335.4933600494533</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A51">
         <v>29</v>
       </c>
-      <c r="B41" s="33">
-        <f>1/5*B37+4/5*B42</f>
+      <c r="B51" s="26">
+        <f>1/5*B47+4/5*B52</f>
         <v>8353.6</v>
       </c>
-      <c r="C41">
-        <f t="shared" si="0"/>
+      <c r="C51">
+        <f t="shared" si="4"/>
         <v>2.275738819632116</v>
       </c>
-      <c r="D41" s="34">
-        <f t="shared" si="1"/>
+      <c r="D51" s="27">
+        <f t="shared" si="5"/>
         <v>2275.7388196321158</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A52">
         <v>30</v>
       </c>
-      <c r="B42">
+      <c r="B52">
         <f>0.7942*10000</f>
         <v>7942</v>
       </c>
-      <c r="C42">
-        <f t="shared" si="0"/>
+      <c r="C52">
+        <f t="shared" si="4"/>
         <v>2.2132426708282242</v>
       </c>
-      <c r="D42" s="34">
-        <f t="shared" si="1"/>
+      <c r="D52" s="27">
+        <f t="shared" si="5"/>
         <v>2213.2426708282242</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A53">
         <v>31</v>
       </c>
-      <c r="B43" s="33">
-        <f>4/5*B42+1/5*B47</f>
+      <c r="B53" s="26">
+        <f>4/5*B52+1/5*B57</f>
         <v>7618.9600000000009</v>
       </c>
-      <c r="C43">
-        <f t="shared" si="0"/>
+      <c r="C53">
+        <f t="shared" si="4"/>
         <v>2.1621480496011118</v>
       </c>
-      <c r="D43" s="34">
-        <f t="shared" si="1"/>
+      <c r="D53" s="27">
+        <f t="shared" si="5"/>
         <v>2162.1480496011118</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A54">
         <v>32</v>
       </c>
-      <c r="B44" s="33">
-        <f>3/5*B42+2/5*B47</f>
+      <c r="B54" s="26">
+        <f>3/5*B52+2/5*B57</f>
         <v>7295.92</v>
       </c>
-      <c r="C44">
-        <f t="shared" si="0"/>
+      <c r="C54">
+        <f t="shared" si="4"/>
         <v>2.1091448156559469</v>
       </c>
-      <c r="D44" s="34">
-        <f t="shared" si="1"/>
+      <c r="D54" s="27">
+        <f t="shared" si="5"/>
         <v>2109.1448156559468</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A55">
         <v>33</v>
       </c>
-      <c r="B45" s="33">
-        <f>2/5*B42+3/5*B47</f>
+      <c r="B55" s="26">
+        <f>2/5*B52+3/5*B57</f>
         <v>6972.88</v>
       </c>
-      <c r="C45">
-        <f t="shared" si="0"/>
+      <c r="C55">
+        <f t="shared" si="4"/>
         <v>2.054123990742879</v>
       </c>
-      <c r="D45" s="34">
-        <f t="shared" si="1"/>
+      <c r="D55" s="27">
+        <f t="shared" si="5"/>
         <v>2054.123990742879</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A56">
         <v>34</v>
       </c>
-      <c r="B46" s="33">
-        <f>1/5*B42+4/5*B47</f>
+      <c r="B56" s="26">
+        <f>1/5*B52+4/5*B57</f>
         <v>6649.84</v>
       </c>
-      <c r="C46">
-        <f t="shared" si="0"/>
+      <c r="C56">
+        <f t="shared" si="4"/>
         <v>1.9969681390331679</v>
       </c>
-      <c r="D46" s="34">
-        <f t="shared" si="1"/>
+      <c r="D56" s="27">
+        <f t="shared" si="5"/>
         <v>1996.968139033168</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A47">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A57">
         <v>35</v>
       </c>
-      <c r="B47">
+      <c r="B57">
         <f>0.63268*10000</f>
         <v>6326.8</v>
       </c>
-      <c r="C47">
-        <f t="shared" si="0"/>
+      <c r="C57">
+        <f t="shared" si="4"/>
         <v>1.9375505304162481</v>
       </c>
-      <c r="D47" s="34">
-        <f t="shared" si="1"/>
+      <c r="D57" s="27">
+        <f t="shared" si="5"/>
         <v>1937.5505304162482</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A48">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A58">
         <v>36</v>
       </c>
-      <c r="B48" s="33">
-        <f>4/5*B47+1/5*B52</f>
+      <c r="B58" s="26">
+        <f>4/5*B57+1/5*B62</f>
         <v>6076.2400000000007</v>
       </c>
-      <c r="C48">
-        <f t="shared" si="0"/>
+      <c r="C58">
+        <f t="shared" si="4"/>
         <v>1.8898200076634835</v>
       </c>
-      <c r="D48" s="34">
-        <f t="shared" si="1"/>
+      <c r="D58" s="27">
+        <f t="shared" si="5"/>
         <v>1889.8200076634835</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A49">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A59">
         <v>37</v>
       </c>
-      <c r="B49" s="33">
-        <f>3/5*B47+2/5*B52</f>
+      <c r="B59" s="26">
+        <f>3/5*B57+2/5*B62</f>
         <v>5825.68</v>
       </c>
-      <c r="C49">
-        <f t="shared" si="0"/>
+      <c r="C59">
+        <f t="shared" si="4"/>
         <v>1.8405780983818707</v>
       </c>
-      <c r="D49" s="34">
-        <f t="shared" si="1"/>
+      <c r="D59" s="27">
+        <f t="shared" si="5"/>
         <v>1840.5780983818706</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A50">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A60">
         <v>38</v>
       </c>
-      <c r="B50" s="33">
-        <f>2/5*B47+3/5*B52</f>
+      <c r="B60" s="26">
+        <f>2/5*B57+3/5*B62</f>
         <v>5575.1200000000008</v>
       </c>
-      <c r="C50">
-        <f t="shared" si="0"/>
+      <c r="C60">
+        <f t="shared" si="4"/>
         <v>1.7897518606598217</v>
       </c>
-      <c r="D50" s="34">
-        <f t="shared" si="1"/>
+      <c r="D60" s="27">
+        <f t="shared" si="5"/>
         <v>1789.7518606598217</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A61">
         <v>39</v>
       </c>
-      <c r="B51" s="33">
-        <f>1/5*B47+4/5*B52</f>
+      <c r="B61" s="26">
+        <f>1/5*B57+4/5*B62</f>
         <v>5324.56</v>
       </c>
-      <c r="C51">
-        <f t="shared" si="0"/>
+      <c r="C61">
+        <f t="shared" si="4"/>
         <v>1.7372635821191604</v>
       </c>
-      <c r="D51" s="34">
-        <f t="shared" si="1"/>
+      <c r="D61" s="27">
+        <f t="shared" si="5"/>
         <v>1737.2635821191604</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A52">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A62">
         <v>40</v>
       </c>
-      <c r="B52">
+      <c r="B62">
         <f>0.5074*10000</f>
         <v>5074</v>
       </c>
-      <c r="C52">
-        <f t="shared" si="0"/>
+      <c r="C62">
+        <f t="shared" si="4"/>
         <v>1.6830303834416878</v>
       </c>
-      <c r="D52" s="34">
-        <f t="shared" si="1"/>
+      <c r="D62" s="27">
+        <f t="shared" si="5"/>
         <v>1683.0303834416877</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A53">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A63">
         <v>41</v>
       </c>
-      <c r="B53" s="33">
-        <f>4/5*B52+1/5*B57</f>
+      <c r="B63" s="26">
+        <f>4/5*B62+1/5*B67</f>
         <v>4879.72</v>
       </c>
-      <c r="C53">
-        <f t="shared" si="0"/>
+      <c r="C63">
+        <f t="shared" si="4"/>
         <v>1.6397217151935652</v>
       </c>
-      <c r="D53" s="34">
-        <f t="shared" si="1"/>
+      <c r="D63" s="27">
+        <f t="shared" si="5"/>
         <v>1639.7217151935652</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A54">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A64">
         <v>42</v>
       </c>
-      <c r="B54" s="33">
-        <f>3/5*B52+2/5*B57</f>
+      <c r="B64" s="26">
+        <f>3/5*B62+2/5*B67</f>
         <v>4685.4400000000005</v>
       </c>
-      <c r="C54">
-        <f t="shared" si="0"/>
+      <c r="C64">
+        <f t="shared" si="4"/>
         <v>1.595267148958424</v>
       </c>
-      <c r="D54" s="34">
-        <f t="shared" si="1"/>
+      <c r="D64" s="27">
+        <f t="shared" si="5"/>
         <v>1595.2671489584241</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A55">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A65">
         <v>43</v>
       </c>
-      <c r="B55" s="33">
-        <f>2/5*B52+3/5*B57</f>
+      <c r="B65" s="26">
+        <f>2/5*B62+3/5*B67</f>
         <v>4491.16</v>
       </c>
-      <c r="C55">
-        <f t="shared" si="0"/>
+      <c r="C65">
+        <f t="shared" si="4"/>
         <v>1.549620596280767</v>
       </c>
-      <c r="D55" s="34">
-        <f t="shared" si="1"/>
+      <c r="D65" s="27">
+        <f t="shared" si="5"/>
         <v>1549.6205962807669</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A56">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A66">
         <v>44</v>
       </c>
-      <c r="B56" s="33">
-        <f>1/5*B52+4/5*B57</f>
+      <c r="B66" s="26">
+        <f>1/5*B62+4/5*B67</f>
         <v>4296.88</v>
       </c>
-      <c r="C56">
-        <f t="shared" si="0"/>
+      <c r="C66">
+        <f t="shared" si="4"/>
         <v>1.502733463524909</v>
       </c>
-      <c r="D56" s="34">
-        <f t="shared" si="1"/>
+      <c r="D66" s="27">
+        <f t="shared" si="5"/>
         <v>1502.733463524909</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A57">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A67">
         <v>45</v>
       </c>
-      <c r="B57">
+      <c r="B67">
         <f>0.41026*10000</f>
         <v>4102.6000000000004</v>
       </c>
-      <c r="C57">
-        <f t="shared" si="0"/>
+      <c r="C67">
+        <f t="shared" si="4"/>
         <v>1.4545544793158709</v>
       </c>
-      <c r="D57" s="34">
-        <f t="shared" si="1"/>
+      <c r="D67" s="27">
+        <f t="shared" si="5"/>
         <v>1454.5544793158708</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A58">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A68">
         <v>46</v>
       </c>
-      <c r="B58" s="33">
-        <f>4/5*B57+1/5*B62</f>
+      <c r="B68" s="26">
+        <f>4/5*B67+1/5*B72</f>
         <v>3949.34</v>
       </c>
-      <c r="C58">
-        <f t="shared" si="0"/>
+      <c r="C68">
+        <f t="shared" si="4"/>
         <v>1.4156010248513551</v>
       </c>
-      <c r="D58" s="34">
-        <f t="shared" si="1"/>
+      <c r="D68" s="27">
+        <f t="shared" si="5"/>
         <v>1415.6010248513551</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A59">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A69">
         <v>47</v>
       </c>
-      <c r="B59" s="33">
-        <f>3/5*B57+2/5*B62</f>
+      <c r="B69" s="26">
+        <f>3/5*B67+2/5*B72</f>
         <v>3796.08</v>
       </c>
-      <c r="C59">
-        <f t="shared" si="0"/>
+      <c r="C69">
+        <f t="shared" si="4"/>
         <v>1.3757821062214772</v>
       </c>
-      <c r="D59" s="34">
-        <f t="shared" si="1"/>
+      <c r="D69" s="27">
+        <f t="shared" si="5"/>
         <v>1375.7821062214773</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A60">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A70">
         <v>48</v>
       </c>
-      <c r="B60" s="33">
-        <f>2/5*B57+3/5*B62</f>
+      <c r="B70" s="26">
+        <f>2/5*B67+3/5*B72</f>
         <v>3642.8199999999997</v>
       </c>
-      <c r="C60">
-        <f t="shared" si="0"/>
+      <c r="C70">
+        <f t="shared" si="4"/>
         <v>1.3350685562075877</v>
       </c>
-      <c r="D60" s="34">
-        <f t="shared" si="1"/>
+      <c r="D70" s="27">
+        <f t="shared" si="5"/>
         <v>1335.0685562075878</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A61">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A71">
         <v>49</v>
       </c>
-      <c r="B61" s="33">
-        <f>1/5*B57+4/5*B62</f>
+      <c r="B71" s="26">
+        <f>1/5*B67+4/5*B72</f>
         <v>3489.56</v>
       </c>
-      <c r="C61">
-        <f t="shared" si="0"/>
+      <c r="C71">
+        <f t="shared" si="4"/>
         <v>1.2934298820717651</v>
       </c>
-      <c r="D61" s="34">
-        <f t="shared" si="1"/>
+      <c r="D71" s="27">
+        <f t="shared" si="5"/>
         <v>1293.4298820717652</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A62">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A72">
         <v>50</v>
       </c>
-      <c r="B62">
+      <c r="B72">
         <f>0.33363*10000</f>
         <v>3336.2999999999997</v>
       </c>
-      <c r="C62">
-        <f t="shared" si="0"/>
+      <c r="C72">
+        <f t="shared" si="4"/>
         <v>1.2508341893928601</v>
       </c>
-      <c r="D62" s="34">
-        <f t="shared" si="1"/>
+      <c r="D72" s="27">
+        <f t="shared" si="5"/>
         <v>1250.83418939286</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A63">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A73">
         <v>51</v>
       </c>
-      <c r="B63" s="33">
-        <f>4/5*B62+1/5*B67</f>
+      <c r="B73" s="26">
+        <f>4/5*B72+1/5*B77</f>
         <v>3213.9</v>
       </c>
-      <c r="C63">
-        <f t="shared" si="0"/>
+      <c r="C73">
+        <f t="shared" si="4"/>
         <v>1.2161057674115894</v>
       </c>
-      <c r="D63" s="34">
-        <f t="shared" si="1"/>
+      <c r="D73" s="27">
+        <f t="shared" si="5"/>
         <v>1216.1057674115893</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A64">
+    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A74">
         <v>52</v>
       </c>
-      <c r="B64" s="33">
-        <f>3/5*B62+2/5*B67</f>
+      <c r="B74" s="26">
+        <f>3/5*B72+2/5*B77</f>
         <v>3091.5</v>
       </c>
-      <c r="C64">
-        <f t="shared" si="0"/>
+      <c r="C74">
+        <f t="shared" si="4"/>
         <v>1.1807279532521102</v>
       </c>
-      <c r="D64" s="34">
-        <f t="shared" si="1"/>
+      <c r="D74" s="27">
+        <f t="shared" si="5"/>
         <v>1180.7279532521102</v>
       </c>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A65">
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A75">
         <v>53</v>
       </c>
-      <c r="B65" s="33">
-        <f>2/5*B62+3/5*B67</f>
+      <c r="B75" s="26">
+        <f>2/5*B72+3/5*B77</f>
         <v>2969.1000000000004</v>
       </c>
-      <c r="C65">
-        <f t="shared" si="0"/>
+      <c r="C75">
+        <f t="shared" si="4"/>
         <v>1.1446823603796716</v>
       </c>
-      <c r="D65" s="34">
-        <f t="shared" si="1"/>
+      <c r="D75" s="27">
+        <f t="shared" si="5"/>
         <v>1144.6823603796715</v>
       </c>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A66">
+    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A76">
         <v>54</v>
       </c>
-      <c r="B66" s="33">
-        <f>1/5*B62+4/5*B67</f>
+      <c r="B76" s="26">
+        <f>1/5*B72+4/5*B77</f>
         <v>2846.7</v>
       </c>
-      <c r="C66">
-        <f t="shared" si="0"/>
+      <c r="C76">
+        <f t="shared" si="4"/>
         <v>1.1079499015311325</v>
       </c>
-      <c r="D66" s="34">
-        <f t="shared" si="1"/>
+      <c r="D76" s="27">
+        <f t="shared" si="5"/>
         <v>1107.9499015311326</v>
       </c>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A67">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A77">
         <v>55</v>
       </c>
-      <c r="B67">
+      <c r="B77">
         <f>0.27243*10000</f>
         <v>2724.3</v>
       </c>
-      <c r="C67">
-        <f t="shared" ref="C67:C82" si="2">B67/(B67+10000)*5</f>
+      <c r="C77">
+        <f t="shared" ref="C77:C92" si="6">B77/(B77+10000)*5</f>
         <v>1.0705107550120636</v>
       </c>
-      <c r="D67" s="34">
-        <f t="shared" ref="D67:D82" si="3">C67*1000</f>
+      <c r="D77" s="27">
+        <f t="shared" ref="D77:D92" si="7">C77*1000</f>
         <v>1070.5107550120636</v>
       </c>
     </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A68">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A78">
         <v>56</v>
       </c>
-      <c r="B68" s="33">
-        <f>4/5*B67+1/5*B72</f>
+      <c r="B78" s="26">
+        <f>4/5*B77+1/5*B82</f>
         <v>2626.84</v>
       </c>
-      <c r="C68">
-        <f t="shared" si="2"/>
+      <c r="C78">
+        <f t="shared" si="6"/>
         <v>1.0401810745998208</v>
       </c>
-      <c r="D68" s="34">
-        <f t="shared" si="3"/>
+      <c r="D78" s="27">
+        <f t="shared" si="7"/>
         <v>1040.1810745998207</v>
       </c>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A69">
+    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A79">
         <v>57</v>
       </c>
-      <c r="B69" s="33">
-        <f>3/5*B67+2/5*B72</f>
+      <c r="B79" s="26">
+        <f>3/5*B77+2/5*B82</f>
         <v>2529.38</v>
       </c>
-      <c r="C69">
-        <f t="shared" si="2"/>
+      <c r="C79">
+        <f t="shared" si="6"/>
         <v>1.0093795542955837</v>
       </c>
-      <c r="D69" s="34">
-        <f t="shared" si="3"/>
+      <c r="D79" s="27">
+        <f t="shared" si="7"/>
         <v>1009.3795542955837</v>
       </c>
     </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A70">
+    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A80">
         <v>58</v>
       </c>
-      <c r="B70" s="33">
-        <f>2/5*B67+3/5*B72</f>
+      <c r="B80" s="26">
+        <f>2/5*B77+3/5*B82</f>
         <v>2431.92</v>
       </c>
-      <c r="C70">
-        <f t="shared" si="2"/>
+      <c r="C80">
+        <f t="shared" si="6"/>
         <v>0.97809509713704723</v>
       </c>
-      <c r="D70" s="34">
-        <f t="shared" si="3"/>
+      <c r="D80" s="27">
+        <f t="shared" si="7"/>
         <v>978.09509713704722</v>
       </c>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A71">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A81">
         <v>59</v>
       </c>
-      <c r="B71" s="33">
-        <f>1/5*B67+4/5*B72</f>
+      <c r="B81" s="26">
+        <f>1/5*B77+4/5*B82</f>
         <v>2334.46</v>
       </c>
-      <c r="C71">
-        <f t="shared" si="2"/>
+      <c r="C81">
+        <f t="shared" si="6"/>
         <v>0.94631625543396314</v>
       </c>
-      <c r="D71" s="34">
-        <f t="shared" si="3"/>
+      <c r="D81" s="27">
+        <f t="shared" si="7"/>
         <v>946.31625543396319</v>
       </c>
     </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A72">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A82">
         <v>60</v>
       </c>
-      <c r="B72">
+      <c r="B82">
         <f>0.2237*10000</f>
         <v>2237</v>
       </c>
-      <c r="C72">
-        <f t="shared" si="2"/>
+      <c r="C82">
+        <f t="shared" si="6"/>
         <v>0.91403121680150368</v>
       </c>
-      <c r="D72" s="34">
-        <f t="shared" si="3"/>
+      <c r="D82" s="27">
+        <f t="shared" si="7"/>
         <v>914.03121680150366</v>
       </c>
     </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A73">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A83">
         <v>61</v>
       </c>
-      <c r="B73" s="33">
-        <f>4/5*B72+1/5*B77</f>
+      <c r="B83" s="26">
+        <f>4/5*B82+1/5*B87</f>
         <v>2158.7800000000002</v>
       </c>
-      <c r="C73">
-        <f t="shared" si="2"/>
+      <c r="C83">
+        <f t="shared" si="6"/>
         <v>0.88774531655314115</v>
       </c>
-      <c r="D73" s="34">
-        <f t="shared" si="3"/>
+      <c r="D83" s="27">
+        <f t="shared" si="7"/>
         <v>887.74531655314115</v>
       </c>
     </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A74">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A84">
         <v>62</v>
       </c>
-      <c r="B74" s="33">
-        <f>3/5*B72+2/5*B77</f>
+      <c r="B84" s="26">
+        <f>3/5*B82+2/5*B87</f>
         <v>2080.5600000000004</v>
       </c>
-      <c r="C74">
-        <f t="shared" si="2"/>
+      <c r="C84">
+        <f t="shared" si="6"/>
         <v>0.86111902097253779</v>
       </c>
-      <c r="D74" s="34">
-        <f t="shared" si="3"/>
+      <c r="D84" s="27">
+        <f t="shared" si="7"/>
         <v>861.11902097253778</v>
       </c>
     </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A75">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A85">
         <v>63</v>
       </c>
-      <c r="B75" s="33">
-        <f>2/5*B72+3/5*B77</f>
+      <c r="B85" s="26">
+        <f>2/5*B82+3/5*B87</f>
         <v>2002.3400000000001</v>
       </c>
-      <c r="C75">
-        <f t="shared" si="2"/>
+      <c r="C85">
+        <f t="shared" si="6"/>
         <v>0.83414567492672276</v>
       </c>
-      <c r="D75" s="34">
-        <f t="shared" si="3"/>
+      <c r="D85" s="27">
+        <f t="shared" si="7"/>
         <v>834.14567492672279</v>
       </c>
     </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A76">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A86">
         <v>64</v>
       </c>
-      <c r="B76" s="33">
-        <f>1/5*B72+4/5*B77</f>
+      <c r="B86" s="26">
+        <f>1/5*B82+4/5*B87</f>
         <v>1924.1200000000003</v>
       </c>
-      <c r="C76">
-        <f t="shared" si="2"/>
+      <c r="C86">
+        <f t="shared" si="6"/>
         <v>0.80681844865700791</v>
       </c>
-      <c r="D76" s="34">
-        <f t="shared" si="3"/>
+      <c r="D86" s="27">
+        <f t="shared" si="7"/>
         <v>806.81844865700793</v>
       </c>
     </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A77">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A87">
         <v>65</v>
       </c>
-      <c r="B77">
+      <c r="B87">
         <f>0.18459*10000</f>
         <v>1845.9</v>
       </c>
-      <c r="C77">
-        <f t="shared" si="2"/>
+      <c r="C87">
+        <f t="shared" si="6"/>
         <v>0.77913033201360804</v>
       </c>
-      <c r="D77" s="34">
-        <f t="shared" si="3"/>
+      <c r="D87" s="27">
+        <f t="shared" si="7"/>
         <v>779.13033201360804</v>
       </c>
     </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A78">
+    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A88">
         <v>66</v>
       </c>
-      <c r="B78" s="33">
-        <f>4/5*B77+1/5*B82</f>
+      <c r="B88" s="26">
+        <f>4/5*B87+1/5*B92</f>
         <v>1782.8200000000002</v>
       </c>
-      <c r="C78">
-        <f t="shared" si="2"/>
+      <c r="C88">
+        <f t="shared" si="6"/>
         <v>0.75653366511582121</v>
       </c>
-      <c r="D78" s="34">
-        <f t="shared" si="3"/>
+      <c r="D88" s="27">
+        <f t="shared" si="7"/>
         <v>756.53366511582124</v>
       </c>
     </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A79">
+    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A89">
         <v>67</v>
       </c>
-      <c r="B79" s="33">
-        <f>3/5*B77+2/5*B82</f>
+      <c r="B89" s="26">
+        <f>3/5*B87+2/5*B92</f>
         <v>1719.74</v>
       </c>
-      <c r="C79">
-        <f t="shared" si="2"/>
+      <c r="C89">
+        <f t="shared" si="6"/>
         <v>0.73369375088525857</v>
       </c>
-      <c r="D79" s="34">
-        <f t="shared" si="3"/>
+      <c r="D89" s="27">
+        <f t="shared" si="7"/>
         <v>733.69375088525862</v>
       </c>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A80">
+    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A90">
         <v>68</v>
       </c>
-      <c r="B80" s="33">
-        <f>2/5*B77+3/5*B82</f>
+      <c r="B90" s="26">
+        <f>2/5*B87+3/5*B92</f>
         <v>1656.66</v>
       </c>
-      <c r="C80">
-        <f t="shared" si="2"/>
+      <c r="C90">
+        <f t="shared" si="6"/>
         <v>0.71060664032407228</v>
       </c>
-      <c r="D80" s="34">
-        <f t="shared" si="3"/>
+      <c r="D90" s="27">
+        <f t="shared" si="7"/>
         <v>710.60664032407226</v>
       </c>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A81">
+    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A91">
         <v>69</v>
       </c>
-      <c r="B81" s="33">
-        <f>1/5*B77+4/5*B82</f>
+      <c r="B91" s="26">
+        <f>1/5*B87+4/5*B92</f>
         <v>1593.5800000000002</v>
       </c>
-      <c r="C81">
-        <f t="shared" si="2"/>
+      <c r="C91">
+        <f t="shared" si="6"/>
         <v>0.68726829848933635</v>
       </c>
-      <c r="D81" s="34">
-        <f t="shared" si="3"/>
+      <c r="D91" s="27">
+        <f t="shared" si="7"/>
         <v>687.2682984893363</v>
       </c>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A82">
+    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A92">
         <v>70</v>
       </c>
-      <c r="B82">
+      <c r="B92">
         <f>0.15305*10000</f>
         <v>1530.5</v>
       </c>
-      <c r="C82">
-        <f t="shared" si="2"/>
+      <c r="C92">
+        <f t="shared" si="6"/>
         <v>0.66367460214214469</v>
       </c>
-      <c r="D82" s="34">
-        <f t="shared" si="3"/>
+      <c r="D92" s="27">
+        <f t="shared" si="7"/>
         <v>663.67460214214464</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A93">
+        <v>71</v>
+      </c>
+      <c r="B93" s="26">
+        <f>4/5*B92+1/5*B97</f>
+        <v>1479.5</v>
+      </c>
+      <c r="C93">
+        <f t="shared" ref="C93:C97" si="8">B93/(B93+10000)*5</f>
+        <v>0.64440959972124223</v>
+      </c>
+      <c r="D93" s="27">
+        <f t="shared" ref="D93:D97" si="9">C93*1000</f>
+        <v>644.40959972124222</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A94">
+        <v>72</v>
+      </c>
+      <c r="B94" s="26">
+        <f>3/5*B92+2/5*B97</f>
+        <v>1428.5</v>
+      </c>
+      <c r="C94">
+        <f t="shared" si="8"/>
+        <v>0.62497265607910046</v>
+      </c>
+      <c r="D94" s="27">
+        <f t="shared" si="9"/>
+        <v>624.97265607910049</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A95">
+        <v>73</v>
+      </c>
+      <c r="B95" s="26">
+        <f>2/5*B92+3/5*B97</f>
+        <v>1377.5</v>
+      </c>
+      <c r="C95">
+        <f t="shared" si="8"/>
+        <v>0.60536145901999561</v>
+      </c>
+      <c r="D95" s="27">
+        <f t="shared" si="9"/>
+        <v>605.36145901999566</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A96">
+        <v>74</v>
+      </c>
+      <c r="B96" s="26">
+        <f>1/5*B92+4/5*B97</f>
+        <v>1326.5</v>
+      </c>
+      <c r="C96">
+        <f t="shared" si="8"/>
+        <v>0.58557365470357126</v>
+      </c>
+      <c r="D96" s="27">
+        <f t="shared" si="9"/>
+        <v>585.57365470357126</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A97">
+        <v>75</v>
+      </c>
+      <c r="B97">
+        <v>1275.5</v>
+      </c>
+      <c r="C97">
+        <f t="shared" si="8"/>
+        <v>0.56560684670302863</v>
+      </c>
+      <c r="D97" s="27">
+        <f t="shared" si="9"/>
+        <v>565.60684670302862</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A98">
+        <v>76</v>
+      </c>
+      <c r="B98" s="26">
+        <f>4/5*B97+1/5*B102</f>
+        <v>1233.94</v>
+      </c>
+      <c r="C98">
+        <f t="shared" ref="C98:C102" si="10">B98/(B98+10000)*5</f>
+        <v>0.54920179384970902</v>
+      </c>
+      <c r="D98" s="27">
+        <f t="shared" ref="D98:D102" si="11">C98*1000</f>
+        <v>549.20179384970902</v>
+      </c>
+    </row>
+    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A99">
+        <v>77</v>
+      </c>
+      <c r="B99" s="26">
+        <f>3/5*B97+2/5*B102</f>
+        <v>1192.3800000000001</v>
+      </c>
+      <c r="C99">
+        <f t="shared" si="10"/>
+        <v>0.53267490917928084</v>
+      </c>
+      <c r="D99" s="27">
+        <f t="shared" si="11"/>
+        <v>532.6749091792808</v>
+      </c>
+    </row>
+    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A100">
+        <v>78</v>
+      </c>
+      <c r="B100" s="26">
+        <f>2/5*B97+3/5*B102</f>
+        <v>1150.8200000000002</v>
+      </c>
+      <c r="C100">
+        <f t="shared" si="10"/>
+        <v>0.51602483046089898</v>
+      </c>
+      <c r="D100" s="27">
+        <f t="shared" si="11"/>
+        <v>516.02483046089901</v>
+      </c>
+    </row>
+    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A101">
+        <v>79</v>
+      </c>
+      <c r="B101" s="26">
+        <f>1/5*B97+4/5*B102</f>
+        <v>1109.2600000000002</v>
+      </c>
+      <c r="C101">
+        <f t="shared" si="10"/>
+        <v>0.4992501750791683</v>
+      </c>
+      <c r="D101" s="27">
+        <f t="shared" si="11"/>
+        <v>499.25017507916829</v>
+      </c>
+    </row>
+    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A102">
+        <v>80</v>
+      </c>
+      <c r="B102">
+        <v>1067.7</v>
+      </c>
+      <c r="C102">
+        <f t="shared" si="10"/>
+        <v>0.48234953965141814</v>
+      </c>
+      <c r="D102" s="27">
+        <f t="shared" si="11"/>
+        <v>482.34953965141813</v>
       </c>
     </row>
   </sheetData>

</xml_diff>